<commit_message>
sml chngs linal session task
</commit_message>
<xml_diff>
--- a/Edu/Linear_algebra/linal_session_task.xlsx
+++ b/Edu/Linear_algebra/linal_session_task.xlsx
@@ -5,16 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iTonyJah\DataScience\Edu\Linear_algebra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LysogorA\DataScience\Edu\Linear_algebra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14622D1-950D-4276-8BAF-F21B4B73FF8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F8E7406-2506-41C1-BA10-E37616AD4BB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
   </bookViews>
   <sheets>
-    <sheet name="1" sheetId="1" r:id="rId1"/>
-    <sheet name="2" sheetId="2" r:id="rId2"/>
+    <sheet name="calc" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="81">
   <si>
     <t>Рабочая таблица с данными:</t>
   </si>
@@ -244,9 +243,6 @@
   </si>
   <si>
     <t>1.</t>
-  </si>
-  <si>
-    <t>2.</t>
   </si>
   <si>
     <t>Матрица признаков Х (5х6)</t>
@@ -288,7 +284,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -432,7 +428,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -456,13 +452,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -475,7 +468,9 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{D5C79018-182E-4F9A-AB42-D02B8D90860C}"/>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -497,8 +492,8 @@
       <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="914400" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="TextBox 3">
@@ -540,6 +535,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -604,7 +600,7 @@
                           <a:rPr lang="en-US" sz="1400" b="0" i="1">
                             <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           </a:rPr>
-                          <m:t>-1</m:t>
+                          <m:t>−1</m:t>
                         </m:r>
                       </m:sup>
                     </m:sSup>
@@ -647,7 +643,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="TextBox 3">
@@ -711,8 +707,8 @@
       <xdr:rowOff>158750</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="914400" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="TextBox 4">
@@ -754,6 +750,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -811,7 +808,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="TextBox 4">
@@ -875,8 +872,8 @@
       <xdr:rowOff>177800</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="654050" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="TextBox 5">
@@ -918,6 +915,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -950,7 +948,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="TextBox 5">
@@ -1014,8 +1012,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="546100" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="TextBox 6">
@@ -1057,6 +1055,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1102,7 +1101,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="TextBox 6">
@@ -1166,8 +1165,8 @@
       <xdr:rowOff>171450</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="914400" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -1209,6 +1208,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1266,7 +1266,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -1330,8 +1330,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="546100" cy="210507"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="TextBox 8">
@@ -1373,6 +1373,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1405,7 +1406,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="TextBox 8">
@@ -1481,8 +1482,8 @@
       <xdr:rowOff>177800</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="546100" cy="209550"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="TextBox 12">
@@ -1524,6 +1525,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1563,7 +1565,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="TextBox 12">
@@ -1627,8 +1629,8 @@
       <xdr:rowOff>165100</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="546100" cy="177800"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="14" name="TextBox 13">
@@ -1670,6 +1672,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1715,7 +1718,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="14" name="TextBox 13">
@@ -1779,8 +1782,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="546100" cy="209550"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="TextBox 14">
@@ -1822,6 +1825,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1861,7 +1865,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="TextBox 14">
@@ -1925,8 +1929,8 @@
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="546100" cy="190500"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="17" name="TextBox 16">
@@ -1968,6 +1972,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1988,7 +1993,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="17" name="TextBox 16">
@@ -2052,8 +2057,8 @@
       <xdr:rowOff>165100</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="596900" cy="203200"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="26" name="TextBox 25">
@@ -2095,6 +2100,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2152,7 +2158,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="26" name="TextBox 25">
@@ -2216,8 +2222,8 @@
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1431353" cy="221214"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="31" name="TextBox 30">
@@ -2259,6 +2265,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2377,7 +2384,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="31" name="TextBox 30">
@@ -2441,8 +2448,8 @@
       <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="991875" cy="461345"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="32" name="TextBox 31">
@@ -2484,6 +2491,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2646,7 +2654,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="32" name="TextBox 31">
@@ -2695,1730 +2703,6 @@
                 <a:t>(𝑥_𝑠𝑡 ) ⃗=(𝑥_𝑐𝑒𝑛𝑡 ) ⃗/(\|(𝑥_𝑐𝑒𝑛𝑡 ) ⃗\|)</a:t>
               </a:r>
               <a:endParaRPr lang="ru-RU" sz="1100"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>25400</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="914400" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2" name="TextBox 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{929052F3-C66C-4F86-8233-773967A1B565}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="25400" y="2533650"/>
-              <a:ext cx="914400" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>(</m:t>
-                        </m:r>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>)</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>-1</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑌</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2" name="TextBox 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{929052F3-C66C-4F86-8233-773967A1B565}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="25400" y="2533650"/>
-              <a:ext cx="914400" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>〖(𝑋〗^𝑇 〖𝑋)〗^(-1) 𝑋^𝑇 𝑌</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>374650</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>158750</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="914400" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="3" name="TextBox 2">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0D48B6F-E69B-46F6-980C-4DA63F9FB042}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="2203450" y="4387850"/>
-              <a:ext cx="914400" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>(</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑋𝑌</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>)</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="3" name="TextBox 2">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0D48B6F-E69B-46F6-980C-4DA63F9FB042}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="2203450" y="4387850"/>
-              <a:ext cx="914400" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑋^𝑇 (𝑋𝑌)</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="654050" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="4" name="TextBox 3">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6943E3A2-EB3E-4BBE-A59D-2C64BE30F571}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="2952750" y="4775200"/>
-              <a:ext cx="654050" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑢</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>=</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑋𝑌</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="4" name="TextBox 3">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6943E3A2-EB3E-4BBE-A59D-2C64BE30F571}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="2952750" y="4775200"/>
-              <a:ext cx="654050" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑢=𝑋𝑌</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="546100" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="5" name="TextBox 4">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0ECADD3-9A6F-4549-9EC1-91A86F3AF6D2}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="4267200" y="4781550"/>
-              <a:ext cx="546100" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑢</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="5" name="TextBox 4">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E0ECADD3-9A6F-4549-9EC1-91A86F3AF6D2}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="4267200" y="4781550"/>
-              <a:ext cx="546100" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑋^𝑇 𝑢</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>355600</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>171450</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="914400" cy="228600"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="6" name="TextBox 5">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{718B0606-25A2-4171-807E-88FA812B1EEB}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="2794000" y="5137150"/>
-              <a:ext cx="914400" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑀</m:t>
-                        </m:r>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>=</m:t>
-                        </m:r>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑋</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="6" name="TextBox 5">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{718B0606-25A2-4171-807E-88FA812B1EEB}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="2794000" y="5137150"/>
-              <a:ext cx="914400" cy="228600"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>〖𝑀=𝑋〗^𝑇 𝑋</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="546100" cy="210507"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="7" name="TextBox 6">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81E014EF-31B1-460A-9580-4F8ADB5678C0}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="4267200" y="5149850"/>
-              <a:ext cx="546100" cy="210507"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:solidFill>
-                          <a:schemeClr val="tx1"/>
-                        </a:solidFill>
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        <a:ea typeface="+mn-ea"/>
-                        <a:cs typeface="+mn-cs"/>
-                      </a:rPr>
-                      <m:t>𝑀𝑌</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" b="0" i="1">
-                <a:solidFill>
-                  <a:schemeClr val="tx1"/>
-                </a:solidFill>
-                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:endParaRPr>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="7" name="TextBox 6">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{81E014EF-31B1-460A-9580-4F8ADB5678C0}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="4267200" y="5149850"/>
-              <a:ext cx="546100" cy="210507"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:rPr>
-                <a:t>𝑀𝑌</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" b="0" i="1">
-                <a:solidFill>
-                  <a:schemeClr val="tx1"/>
-                </a:solidFill>
-                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:endParaRPr>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="546100" cy="209550"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="8" name="TextBox 7">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C01BE8A9-A19D-46B2-9E64-7EDC1BDCBC4B}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="3657600" y="7924800"/>
-              <a:ext cx="546100" cy="209550"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="8" name="TextBox 7">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C01BE8A9-A19D-46B2-9E64-7EDC1BDCBC4B}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="3657600" y="7924800"/>
-              <a:ext cx="546100" cy="209550"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑋^𝑇</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="546100" cy="177800"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="9" name="TextBox 8">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{746C753A-AAE2-4D49-A996-E1949D6FEA0A}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="0" y="7912100"/>
-              <a:ext cx="546100" cy="177800"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑢</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="9" name="TextBox 8">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{746C753A-AAE2-4D49-A996-E1949D6FEA0A}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="0" y="7912100"/>
-              <a:ext cx="546100" cy="177800"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑋^𝑇 𝑢</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>49</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="546100" cy="209550"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="10" name="TextBox 9">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0DDCD70-35D5-46BD-AB10-C7EA98BB39C2}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="3695700" y="9220200"/>
-              <a:ext cx="546100" cy="209550"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="10" name="TextBox 9">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0DDCD70-35D5-46BD-AB10-C7EA98BB39C2}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="3695700" y="9220200"/>
-              <a:ext cx="546100" cy="209550"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑋^𝑇</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>59</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="546100" cy="190500"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="11" name="TextBox 10">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDE7F6EA-57FD-4F2B-BA74-9E7734625934}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="0" y="11214100"/>
-              <a:ext cx="546100" cy="190500"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑀𝑌</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="11" name="TextBox 10">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDE7F6EA-57FD-4F2B-BA74-9E7734625934}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="0" y="11214100"/>
-              <a:ext cx="546100" cy="190500"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑀𝑌</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>6350</xdr:colOff>
-      <xdr:row>66</xdr:row>
-      <xdr:rowOff>165100</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="596900" cy="203200"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="12" name="TextBox 11">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D44DF6A-3904-42AD-9DE7-5B51625B8468}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="6350" y="12515850"/>
-              <a:ext cx="596900" cy="203200"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑋</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>𝑇</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>(</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>𝑋𝑌</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1400" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>)</m:t>
-                    </m:r>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="12" name="TextBox 11">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D44DF6A-3904-42AD-9DE7-5B51625B8468}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="6350" y="12515850"/>
-              <a:ext cx="596900" cy="203200"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:noAutofit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-US" sz="1400" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑋^𝑇 (𝑋𝑌)</a:t>
-              </a:r>
-              <a:endParaRPr lang="ru-RU" sz="1400" i="1"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
@@ -4747,14 +3031,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472F5A48-0D57-45D1-AF67-58628EB4925B}">
   <dimension ref="A1:L109"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -4777,7 +3061,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>3</v>
       </c>
@@ -4800,7 +3084,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -4823,7 +3107,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>2</v>
       </c>
@@ -4846,7 +3130,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>3</v>
       </c>
@@ -4869,7 +3153,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>1</v>
       </c>
@@ -4892,32 +3176,32 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="23" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:7" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -4925,7 +3209,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>3</v>
       </c>
@@ -4939,7 +3223,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>1</v>
       </c>
@@ -4953,7 +3237,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>2</v>
       </c>
@@ -4967,22 +3251,22 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>19</v>
       </c>
@@ -4990,12 +3274,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -5003,42 +3287,42 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="16" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>28</v>
       </c>
@@ -5049,7 +3333,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="7">
         <f>F38*J$38+G38*J$39+H38*J$40</f>
         <v>93900</v>
@@ -5071,7 +3355,7 @@
       </c>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="7">
         <f t="shared" ref="A39:A40" si="0">F39*J$38+G39*J$39+H39*J$40</f>
         <v>52100</v>
@@ -5093,7 +3377,7 @@
       </c>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
         <f t="shared" si="0"/>
         <v>80200</v>
@@ -5115,23 +3399,23 @@
       </c>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B41" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
       <c r="J43" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="12">
         <f>F44*J$44+G44*J$45+H44*J$46</f>
         <v>494200</v>
@@ -5153,7 +3437,7 @@
       </c>
       <c r="L44" s="8"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="12">
         <f t="shared" ref="A45:A46" si="1">F45*J$44+G45*J$45+H45*J$46</f>
         <v>9960900</v>
@@ -5175,7 +3459,7 @@
       </c>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="12">
         <f t="shared" si="1"/>
         <v>494200</v>
@@ -5197,22 +3481,22 @@
       </c>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B47" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B50" s="6" t="s">
         <v>43</v>
       </c>
@@ -5220,7 +3504,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="12">
         <f>$F51*J$51+$G51*J$52+$H51*J$53</f>
         <v>14</v>
@@ -5252,7 +3536,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="12">
         <f t="shared" ref="A52:A53" si="4">$F52*J$51+$G52*J$52+$H52*J$53</f>
         <v>273</v>
@@ -5284,7 +3568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="12">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -5316,12 +3600,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>38</v>
       </c>
@@ -5332,7 +3616,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="12">
         <f>$F51*J$51+$G51*J$52+$H51*J$53</f>
         <v>14</v>
@@ -5355,7 +3639,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="12">
         <f>$F52*J$51+$G52*J$52+$H52*J$53</f>
         <v>273</v>
@@ -5378,7 +3662,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="12">
         <f>$F53*J$51+$G53*J$52+$H53*J$53</f>
         <v>14</v>
@@ -5401,19 +3685,19 @@
         <v>48</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B59" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>51</v>
       </c>
       <c r="B60" s="8"/>
       <c r="F60" s="8"/>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G61" s="6" t="s">
         <v>43</v>
       </c>
@@ -5421,12 +3705,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="12">
         <f>F62*J$62+G62*J$63+H62*J$64</f>
         <v>494200</v>
       </c>
-      <c r="B62" s="15" t="s">
+      <c r="B62" s="8" t="s">
         <v>53</v>
       </c>
       <c r="F62" s="12">
@@ -5442,12 +3726,12 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="12">
         <f t="shared" ref="A63:A64" si="5">F63*J$62+G63*J$63+H63*J$64</f>
         <v>9960900</v>
       </c>
-      <c r="B63" s="15" t="s">
+      <c r="B63" s="8" t="s">
         <v>52</v>
       </c>
       <c r="F63" s="12">
@@ -5463,12 +3747,12 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="12">
         <f t="shared" si="5"/>
         <v>494200</v>
       </c>
-      <c r="B64" s="15" t="s">
+      <c r="B64" s="8" t="s">
         <v>53</v>
       </c>
       <c r="F64" s="12">
@@ -5484,117 +3768,117 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B65" s="11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B67" s="15"/>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="C68" s="16" t="s">
+      <c r="B67" s="8"/>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C68" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="12">
         <v>494200</v>
       </c>
-      <c r="C69" s="16" t="s">
+      <c r="C69" s="8" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="12">
         <v>9960900</v>
       </c>
-      <c r="C70" s="17" t="s">
+      <c r="C70" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="12">
         <v>494200</v>
       </c>
-      <c r="C71" s="17" t="s">
+      <c r="C71" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="23" x14ac:dyDescent="0.35">
-      <c r="A74" s="18" t="s">
+    <row r="74" spans="1:3" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A74" s="15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>1</v>
       </c>
@@ -5617,19 +3901,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C90" s="19"/>
-      <c r="D90" s="19"/>
-      <c r="E90" s="19" t="s">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="C90" s="16"/>
+      <c r="D90" s="16"/>
+      <c r="E90" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="F90" s="16"/>
+      <c r="G90" s="16"/>
+      <c r="I90" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="F90" s="19"/>
-      <c r="G90" s="19"/>
-      <c r="I90" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B91" s="7">
         <v>3</v>
       </c>
@@ -5652,7 +3936,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B92" s="7">
         <v>1</v>
       </c>
@@ -5675,7 +3959,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B93" s="7">
         <v>2</v>
       </c>
@@ -5698,7 +3982,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B94" s="7">
         <v>3</v>
       </c>
@@ -5721,7 +4005,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B95" s="7">
         <v>1</v>
       </c>
@@ -5744,19 +4028,19 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
-        <v>77</v>
       </c>
       <c r="B99">
         <f>SUM(B91:B95)</f>
@@ -5787,15 +4071,15 @@
         <v>12200</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B100">
         <f>B99/5</f>
         <v>2</v>
       </c>
-      <c r="C100">
+      <c r="C100" s="17">
         <f t="shared" ref="C100:I100" si="7">C99/5</f>
         <v>45.2</v>
       </c>
@@ -5803,11 +4087,11 @@
         <f t="shared" si="7"/>
         <v>2</v>
       </c>
-      <c r="E100">
+      <c r="E100" s="17">
         <f t="shared" si="7"/>
         <v>0.2</v>
       </c>
-      <c r="F100">
+      <c r="F100" s="17">
         <f t="shared" si="7"/>
         <v>0.8</v>
       </c>
@@ -5820,17 +4104,17 @@
         <v>2440</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B102" s="7">
         <f>B91-B$100</f>
         <v>1</v>
       </c>
-      <c r="C102" s="20">
+      <c r="C102" s="17">
         <f t="shared" ref="C102:G102" si="8">C91-C$100</f>
         <v>5.7999999999999972</v>
       </c>
@@ -5838,11 +4122,11 @@
         <f t="shared" si="8"/>
         <v>1</v>
       </c>
-      <c r="E102" s="7">
+      <c r="E102" s="17">
         <f t="shared" si="8"/>
         <v>-0.2</v>
       </c>
-      <c r="F102" s="7">
+      <c r="F102" s="17">
         <f t="shared" si="8"/>
         <v>0.19999999999999996</v>
       </c>
@@ -5855,12 +4139,12 @@
         <v>-240</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B103" s="7">
         <f t="shared" ref="B103:G103" si="10">B92-B$100</f>
         <v>-1</v>
       </c>
-      <c r="C103" s="20">
+      <c r="C103" s="17">
         <f t="shared" si="10"/>
         <v>-15.200000000000003</v>
       </c>
@@ -5868,11 +4152,11 @@
         <f t="shared" si="10"/>
         <v>-1</v>
       </c>
-      <c r="E103" s="7">
+      <c r="E103" s="17">
         <f t="shared" si="10"/>
         <v>-0.2</v>
       </c>
-      <c r="F103" s="7">
+      <c r="F103" s="17">
         <f t="shared" si="10"/>
         <v>0.19999999999999996</v>
       </c>
@@ -5885,12 +4169,12 @@
         <v>-840</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B104" s="7">
         <f t="shared" ref="B104:G104" si="12">B93-B$100</f>
         <v>0</v>
       </c>
-      <c r="C104" s="20">
+      <c r="C104" s="17">
         <f t="shared" si="12"/>
         <v>-0.20000000000000284</v>
       </c>
@@ -5898,11 +4182,11 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="E104" s="7">
+      <c r="E104" s="17">
         <f t="shared" si="12"/>
         <v>-0.2</v>
       </c>
-      <c r="F104" s="7">
+      <c r="F104" s="17">
         <f t="shared" si="12"/>
         <v>0.19999999999999996</v>
       </c>
@@ -5915,12 +4199,12 @@
         <v>-540</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B105" s="7">
         <f t="shared" ref="B105:G105" si="14">B94-B$100</f>
         <v>1</v>
       </c>
-      <c r="C105" s="20">
+      <c r="C105" s="17">
         <f t="shared" si="14"/>
         <v>9.7999999999999972</v>
       </c>
@@ -5928,11 +4212,11 @@
         <f t="shared" si="14"/>
         <v>-1</v>
       </c>
-      <c r="E105" s="7">
+      <c r="E105" s="17">
         <f t="shared" si="14"/>
         <v>-0.2</v>
       </c>
-      <c r="F105" s="7">
+      <c r="F105" s="17">
         <f t="shared" si="14"/>
         <v>0.19999999999999996</v>
       </c>
@@ -5945,12 +4229,12 @@
         <v>-440</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B106" s="7">
         <f t="shared" ref="B106:G106" si="16">B95-B$100</f>
         <v>-1</v>
       </c>
-      <c r="C106" s="20">
+      <c r="C106" s="17">
         <f t="shared" si="16"/>
         <v>-0.20000000000000284</v>
       </c>
@@ -5958,11 +4242,11 @@
         <f t="shared" si="16"/>
         <v>1</v>
       </c>
-      <c r="E106" s="7">
+      <c r="E106" s="17">
         <f t="shared" si="16"/>
         <v>0.8</v>
       </c>
-      <c r="F106" s="7">
+      <c r="F106" s="17">
         <f t="shared" si="16"/>
         <v>-0.8</v>
       </c>
@@ -5975,17 +4259,17 @@
         <v>2060</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A108" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B109">
         <f>(B102^2+B103^2+B104^2+B105^2+B106^2)^(1/2)</f>
         <v>2</v>
@@ -6017,1002 +4301,6 @@
       <c r="I109">
         <f t="shared" si="18"/>
         <v>2343.5016535091245</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D34DEDF-4E36-4037-8F0A-6A5E0D2037C2}">
-  <dimension ref="A1:L94"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2">
-        <v>3</v>
-      </c>
-      <c r="B3" s="2">
-        <v>51</v>
-      </c>
-      <c r="C3" s="2">
-        <v>3</v>
-      </c>
-      <c r="D3" s="2">
-        <v>0</v>
-      </c>
-      <c r="E3" s="2">
-        <v>1</v>
-      </c>
-      <c r="F3" s="2">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="3">
-        <v>1</v>
-      </c>
-      <c r="B4" s="3">
-        <v>30</v>
-      </c>
-      <c r="C4" s="3">
-        <v>1</v>
-      </c>
-      <c r="D4" s="3">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3">
-        <v>0</v>
-      </c>
-      <c r="G4" s="3">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3">
-        <v>2</v>
-      </c>
-      <c r="B5" s="3">
-        <v>45</v>
-      </c>
-      <c r="C5" s="3">
-        <v>2</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0</v>
-      </c>
-      <c r="E5" s="3">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3">
-        <v>0</v>
-      </c>
-      <c r="G5" s="3">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="3">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3">
-        <v>55</v>
-      </c>
-      <c r="C6" s="3">
-        <v>1</v>
-      </c>
-      <c r="D6" s="3">
-        <v>0</v>
-      </c>
-      <c r="E6" s="3">
-        <v>1</v>
-      </c>
-      <c r="F6" s="3">
-        <v>0</v>
-      </c>
-      <c r="G6" s="3">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3">
-        <v>1</v>
-      </c>
-      <c r="B7" s="3">
-        <v>45</v>
-      </c>
-      <c r="C7" s="3">
-        <v>3</v>
-      </c>
-      <c r="D7" s="3">
-        <v>1</v>
-      </c>
-      <c r="E7" s="3">
-        <v>0</v>
-      </c>
-      <c r="F7" s="3">
-        <v>0</v>
-      </c>
-      <c r="G7" s="3">
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="23" x14ac:dyDescent="0.5">
-      <c r="A9" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="C14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="C15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="2">
-        <v>3</v>
-      </c>
-      <c r="B18" s="2">
-        <v>51</v>
-      </c>
-      <c r="C18" s="2">
-        <v>3</v>
-      </c>
-      <c r="E18" s="2">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A19" s="3">
-        <v>1</v>
-      </c>
-      <c r="B19" s="3">
-        <v>30</v>
-      </c>
-      <c r="C19" s="3">
-        <v>1</v>
-      </c>
-      <c r="E19" s="3">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="3">
-        <v>2</v>
-      </c>
-      <c r="B20" s="3">
-        <v>45</v>
-      </c>
-      <c r="C20" s="3">
-        <v>2</v>
-      </c>
-      <c r="E20" s="3">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>19</v>
-      </c>
-      <c r="G26" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" ht="16" x14ac:dyDescent="0.4">
-      <c r="A33" s="14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A37" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="G37" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="J37" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A38" s="7">
-        <f>F38*J$38+G38*J$39+H38*J$40</f>
-        <v>93900</v>
-      </c>
-      <c r="B38" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="F38" s="7">
-        <v>3</v>
-      </c>
-      <c r="G38" s="7">
-        <v>51</v>
-      </c>
-      <c r="H38" s="7">
-        <v>3</v>
-      </c>
-      <c r="J38" s="7">
-        <v>2200</v>
-      </c>
-      <c r="L38" s="8"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A39" s="7">
-        <f t="shared" ref="A39:A40" si="0">F39*J$38+G39*J$39+H39*J$40</f>
-        <v>52100</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F39" s="7">
-        <v>1</v>
-      </c>
-      <c r="G39" s="7">
-        <v>30</v>
-      </c>
-      <c r="H39" s="7">
-        <v>1</v>
-      </c>
-      <c r="J39" s="7">
-        <v>1600</v>
-      </c>
-      <c r="L39" s="8"/>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A40" s="7">
-        <f t="shared" si="0"/>
-        <v>80200</v>
-      </c>
-      <c r="B40" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="F40" s="7">
-        <v>2</v>
-      </c>
-      <c r="G40" s="7">
-        <v>45</v>
-      </c>
-      <c r="H40" s="7">
-        <v>2</v>
-      </c>
-      <c r="J40" s="7">
-        <v>1900</v>
-      </c>
-      <c r="L40" s="8"/>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B41" s="11" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A43" s="10"/>
-      <c r="J43" s="10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A44" s="12">
-        <f>F44*J$44+G44*J$45+H44*J$46</f>
-        <v>494200</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F44" s="7">
-        <v>3</v>
-      </c>
-      <c r="G44" s="7">
-        <v>1</v>
-      </c>
-      <c r="H44" s="7">
-        <v>2</v>
-      </c>
-      <c r="J44" s="12">
-        <v>93900</v>
-      </c>
-      <c r="L44" s="8"/>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A45" s="12">
-        <f t="shared" ref="A45:A46" si="1">F45*J$44+G45*J$45+H45*J$46</f>
-        <v>9960900</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="F45" s="7">
-        <v>51</v>
-      </c>
-      <c r="G45" s="7">
-        <v>30</v>
-      </c>
-      <c r="H45" s="7">
-        <v>45</v>
-      </c>
-      <c r="J45" s="12">
-        <v>52100</v>
-      </c>
-      <c r="L45" s="8"/>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A46" s="12">
-        <f t="shared" si="1"/>
-        <v>494200</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F46" s="7">
-        <v>3</v>
-      </c>
-      <c r="G46" s="7">
-        <v>1</v>
-      </c>
-      <c r="H46" s="7">
-        <v>2</v>
-      </c>
-      <c r="J46" s="12">
-        <v>80200</v>
-      </c>
-      <c r="L46" s="8"/>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B47" s="11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A48" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B50" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="K50" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A51" s="12">
-        <f>$F51*J$51+$G51*J$52+$H51*J$53</f>
-        <v>14</v>
-      </c>
-      <c r="B51" s="12">
-        <f t="shared" ref="B51:C53" si="2">$F51*K$51+$G51*K$52+$H51*K$53</f>
-        <v>273</v>
-      </c>
-      <c r="C51" s="12">
-        <f t="shared" si="2"/>
-        <v>14</v>
-      </c>
-      <c r="F51" s="7">
-        <v>3</v>
-      </c>
-      <c r="G51" s="7">
-        <v>1</v>
-      </c>
-      <c r="H51" s="7">
-        <v>2</v>
-      </c>
-      <c r="J51" s="7">
-        <v>3</v>
-      </c>
-      <c r="K51" s="7">
-        <v>51</v>
-      </c>
-      <c r="L51" s="7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A52" s="12">
-        <f t="shared" ref="A52:A53" si="3">$F52*J$51+$G52*J$52+$H52*J$53</f>
-        <v>273</v>
-      </c>
-      <c r="B52" s="12">
-        <f t="shared" si="2"/>
-        <v>5526</v>
-      </c>
-      <c r="C52" s="12">
-        <f t="shared" si="2"/>
-        <v>273</v>
-      </c>
-      <c r="F52" s="7">
-        <v>51</v>
-      </c>
-      <c r="G52" s="7">
-        <v>30</v>
-      </c>
-      <c r="H52" s="7">
-        <v>45</v>
-      </c>
-      <c r="J52" s="7">
-        <v>1</v>
-      </c>
-      <c r="K52" s="7">
-        <v>30</v>
-      </c>
-      <c r="L52" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A53" s="12">
-        <f t="shared" si="3"/>
-        <v>14</v>
-      </c>
-      <c r="B53" s="12">
-        <f t="shared" si="2"/>
-        <v>273</v>
-      </c>
-      <c r="C53" s="12">
-        <f t="shared" si="2"/>
-        <v>14</v>
-      </c>
-      <c r="F53" s="7">
-        <v>3</v>
-      </c>
-      <c r="G53" s="7">
-        <v>1</v>
-      </c>
-      <c r="H53" s="7">
-        <v>2</v>
-      </c>
-      <c r="J53" s="7">
-        <v>2</v>
-      </c>
-      <c r="K53" s="7">
-        <v>45</v>
-      </c>
-      <c r="L53" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>38</v>
-      </c>
-      <c r="E55" t="s">
-        <v>39</v>
-      </c>
-      <c r="I55" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A56" s="12">
-        <f>$F51*J$51+$G51*J$52+$H51*J$53</f>
-        <v>14</v>
-      </c>
-      <c r="B56" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E56" s="12">
-        <f>$F51*K$51+$G51*K$52+$H51*K$53</f>
-        <v>273</v>
-      </c>
-      <c r="F56" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="I56" s="12">
-        <f>$F51*L$51+$G51*L$52+$H51*L$53</f>
-        <v>14</v>
-      </c>
-      <c r="J56" s="8" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A57" s="12">
-        <f>$F52*J$51+$G52*J$52+$H52*J$53</f>
-        <v>273</v>
-      </c>
-      <c r="B57" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E57" s="12">
-        <f>$F52*K$51+$G52*K$52+$H52*K$53</f>
-        <v>5526</v>
-      </c>
-      <c r="F57" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="I57" s="12">
-        <f>$F52*L$51+$G52*L$52+$H52*L$53</f>
-        <v>273</v>
-      </c>
-      <c r="J57" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A58" s="12">
-        <f>$F53*J$51+$G53*J$52+$H53*J$53</f>
-        <v>14</v>
-      </c>
-      <c r="B58" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="E58" s="12">
-        <f>$F53*K$51+$G53*K$52+$H53*K$53</f>
-        <v>273</v>
-      </c>
-      <c r="F58" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="I58" s="12">
-        <f>$F53*L$51+$G53*L$52+$H53*L$53</f>
-        <v>14</v>
-      </c>
-      <c r="J58" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="B59" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>51</v>
-      </c>
-      <c r="B60" s="8"/>
-      <c r="F60" s="8"/>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="G61" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J61" s="10" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A62" s="12">
-        <f>F62*J$62+G62*J$63+H62*J$64</f>
-        <v>494200</v>
-      </c>
-      <c r="B62" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="F62" s="12">
-        <v>14</v>
-      </c>
-      <c r="G62" s="12">
-        <v>273</v>
-      </c>
-      <c r="H62" s="12">
-        <v>14</v>
-      </c>
-      <c r="J62" s="7">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A63" s="12">
-        <f t="shared" ref="A63:A64" si="4">F63*J$62+G63*J$63+H63*J$64</f>
-        <v>9960900</v>
-      </c>
-      <c r="B63" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="F63" s="12">
-        <v>273</v>
-      </c>
-      <c r="G63" s="12">
-        <v>5526</v>
-      </c>
-      <c r="H63" s="12">
-        <v>273</v>
-      </c>
-      <c r="J63" s="7">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A64" s="12">
-        <f t="shared" si="4"/>
-        <v>494200</v>
-      </c>
-      <c r="B64" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="F64" s="12">
-        <v>14</v>
-      </c>
-      <c r="G64" s="12">
-        <v>273</v>
-      </c>
-      <c r="H64" s="12">
-        <v>14</v>
-      </c>
-      <c r="J64" s="7">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B65" s="11" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A67" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B67" s="15"/>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="C68" s="16" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A69" s="12">
-        <v>494200</v>
-      </c>
-      <c r="C69" s="16" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A70" s="12">
-        <v>9960900</v>
-      </c>
-      <c r="C70" s="17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A71" s="12">
-        <v>494200</v>
-      </c>
-      <c r="C71" s="17" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="23" x14ac:dyDescent="0.35">
-      <c r="A74" s="18" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A75" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A84" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A85" s="13" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
-        <v>1</v>
-      </c>
-      <c r="B86" t="s">
-        <v>2</v>
-      </c>
-      <c r="C86" t="s">
-        <v>3</v>
-      </c>
-      <c r="D86" t="s">
-        <v>4</v>
-      </c>
-      <c r="E86" t="s">
-        <v>5</v>
-      </c>
-      <c r="F86" t="s">
-        <v>6</v>
-      </c>
-      <c r="H86" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B87" s="19"/>
-      <c r="C87" s="19"/>
-      <c r="D87" s="19" t="s">
-        <v>70</v>
-      </c>
-      <c r="E87" s="19"/>
-      <c r="F87" s="19"/>
-      <c r="H87" s="9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A88" s="7">
-        <v>3</v>
-      </c>
-      <c r="B88" s="7">
-        <v>51</v>
-      </c>
-      <c r="C88" s="7">
-        <v>3</v>
-      </c>
-      <c r="D88" s="7">
-        <v>0</v>
-      </c>
-      <c r="E88" s="7">
-        <v>1</v>
-      </c>
-      <c r="F88" s="7">
-        <v>0</v>
-      </c>
-      <c r="H88" s="7">
-        <v>2200</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A89" s="7">
-        <v>1</v>
-      </c>
-      <c r="B89" s="7">
-        <v>30</v>
-      </c>
-      <c r="C89" s="7">
-        <v>1</v>
-      </c>
-      <c r="D89" s="7">
-        <v>0</v>
-      </c>
-      <c r="E89" s="7">
-        <v>1</v>
-      </c>
-      <c r="F89" s="7">
-        <v>0</v>
-      </c>
-      <c r="H89" s="7">
-        <v>1600</v>
-      </c>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A90" s="7">
-        <v>2</v>
-      </c>
-      <c r="B90" s="7">
-        <v>45</v>
-      </c>
-      <c r="C90" s="7">
-        <v>2</v>
-      </c>
-      <c r="D90" s="7">
-        <v>0</v>
-      </c>
-      <c r="E90" s="7">
-        <v>1</v>
-      </c>
-      <c r="F90" s="7">
-        <v>0</v>
-      </c>
-      <c r="H90" s="7">
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A91" s="7">
-        <v>3</v>
-      </c>
-      <c r="B91" s="7">
-        <v>55</v>
-      </c>
-      <c r="C91" s="7">
-        <v>1</v>
-      </c>
-      <c r="D91" s="7">
-        <v>0</v>
-      </c>
-      <c r="E91" s="7">
-        <v>1</v>
-      </c>
-      <c r="F91" s="7">
-        <v>0</v>
-      </c>
-      <c r="H91" s="7">
-        <v>2000</v>
-      </c>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A92" s="7">
-        <v>1</v>
-      </c>
-      <c r="B92" s="7">
-        <v>45</v>
-      </c>
-      <c r="C92" s="7">
-        <v>3</v>
-      </c>
-      <c r="D92" s="7">
-        <v>1</v>
-      </c>
-      <c r="E92" s="7">
-        <v>0</v>
-      </c>
-      <c r="F92" s="7">
-        <v>0</v>
-      </c>
-      <c r="H92" s="7">
-        <v>4500</v>
-      </c>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A94" s="13" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
linal sesion 1st task
</commit_message>
<xml_diff>
--- a/Edu/Linear_algebra/linal_session_task.xlsx
+++ b/Edu/Linear_algebra/linal_session_task.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iTonyJah\DataScience\Edu\Linear_algebra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LysogorA\DataScience\Edu\Linear_algebra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD744CE6-9E45-41B3-ACBB-F1C8780E04B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF331A3A-F6DE-41C8-BBD3-2261C83B749F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
   </bookViews>
   <sheets>
     <sheet name="calc" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="91">
   <si>
     <t>Рабочая таблица с данными:</t>
   </si>
@@ -294,6 +294,21 @@
   </si>
   <si>
     <t>90+14</t>
+  </si>
+  <si>
+    <t>=2^4*3*5</t>
+  </si>
+  <si>
+    <t>=7*5*3*2^3</t>
+  </si>
+  <si>
+    <t>=5*3^3*2^2</t>
+  </si>
+  <si>
+    <t>=11*5*2^3</t>
+  </si>
+  <si>
+    <t>=103*5*2^2</t>
   </si>
 </sst>
 </file>
@@ -490,7 +505,7 @@
     </xf>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3058,18 +3073,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472F5A48-0D57-45D1-AF67-58628EB4925B}">
-  <dimension ref="A1:AD127"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AD136"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="25" max="25" width="12.7265625" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3092,7 +3107,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>3</v>
       </c>
@@ -3115,7 +3130,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -3138,7 +3153,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>2</v>
       </c>
@@ -3161,7 +3176,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>3</v>
       </c>
@@ -3184,7 +3199,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>1</v>
       </c>
@@ -3207,32 +3222,32 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="23" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:7" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -3240,7 +3255,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>3</v>
       </c>
@@ -3254,7 +3269,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>1</v>
       </c>
@@ -3268,7 +3283,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>2</v>
       </c>
@@ -3282,22 +3297,22 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>19</v>
       </c>
@@ -3305,12 +3320,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -3318,42 +3333,42 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="16" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>28</v>
       </c>
@@ -3364,7 +3379,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="7">
         <f>F38*J$38+G38*J$39+H38*J$40</f>
         <v>93900</v>
@@ -3386,7 +3401,7 @@
       </c>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="7">
         <f t="shared" ref="A39:A40" si="0">F39*J$38+G39*J$39+H39*J$40</f>
         <v>52100</v>
@@ -3408,7 +3423,7 @@
       </c>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
         <f t="shared" si="0"/>
         <v>80200</v>
@@ -3430,23 +3445,23 @@
       </c>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B41" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
       <c r="J43" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="12">
         <f>F44*J$44+G44*J$45+H44*J$46</f>
         <v>494200</v>
@@ -3468,7 +3483,7 @@
       </c>
       <c r="L44" s="8"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="12">
         <f t="shared" ref="A45:A46" si="1">F45*J$44+G45*J$45+H45*J$46</f>
         <v>9960900</v>
@@ -3490,7 +3505,7 @@
       </c>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="12">
         <f t="shared" si="1"/>
         <v>494200</v>
@@ -3512,22 +3527,22 @@
       </c>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B47" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B50" s="6" t="s">
         <v>43</v>
       </c>
@@ -3535,7 +3550,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="12">
         <f>$F51*J$51+$G51*J$52+$H51*J$53</f>
         <v>14</v>
@@ -3567,7 +3582,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="12">
         <f t="shared" ref="A52:A53" si="4">$F52*J$51+$G52*J$52+$H52*J$53</f>
         <v>273</v>
@@ -3599,7 +3614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="12">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -3631,12 +3646,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>38</v>
       </c>
@@ -3647,7 +3662,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="12">
         <f>$F51*J$51+$G51*J$52+$H51*J$53</f>
         <v>14</v>
@@ -3670,7 +3685,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="12">
         <f>$F52*J$51+$G52*J$52+$H52*J$53</f>
         <v>273</v>
@@ -3693,7 +3708,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="12">
         <f>$F53*J$51+$G53*J$52+$H53*J$53</f>
         <v>14</v>
@@ -3716,19 +3731,19 @@
         <v>48</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B59" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>51</v>
       </c>
       <c r="B60" s="8"/>
       <c r="F60" s="8"/>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G61" s="6" t="s">
         <v>43</v>
       </c>
@@ -3736,7 +3751,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="12">
         <f>F62*J$62+G62*J$63+H62*J$64</f>
         <v>494200</v>
@@ -3757,7 +3772,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="12">
         <f t="shared" ref="A63:A64" si="5">F63*J$62+G63*J$63+H63*J$64</f>
         <v>9960900</v>
@@ -3778,7 +3793,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="12">
         <f t="shared" si="5"/>
         <v>494200</v>
@@ -3799,23 +3814,23 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B65" s="11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B67" s="8"/>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C68" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="12">
         <v>494200</v>
       </c>
@@ -3823,7 +3838,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="12">
         <v>9960900</v>
       </c>
@@ -3831,7 +3846,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="12">
         <v>494200</v>
       </c>
@@ -3839,77 +3854,77 @@
         <v>59</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="23" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>1</v>
       </c>
@@ -3932,7 +3947,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C90" s="16"/>
       <c r="D90" s="16"/>
       <c r="E90" s="16" t="s">
@@ -3944,7 +3959,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B91" s="7">
         <v>3</v>
       </c>
@@ -3967,7 +3982,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B92" s="7">
         <v>1</v>
       </c>
@@ -3990,7 +4005,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B93" s="7">
         <v>2</v>
       </c>
@@ -4013,7 +4028,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B94" s="7">
         <v>3</v>
       </c>
@@ -4036,7 +4051,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B95" s="7">
         <v>1</v>
       </c>
@@ -4059,17 +4074,17 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="97" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="13" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="98" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="99" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>76</v>
       </c>
@@ -4112,7 +4127,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="100" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>77</v>
       </c>
@@ -4149,7 +4164,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="101" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>78</v>
       </c>
@@ -4166,7 +4181,7 @@
         <v>0.44721359549995798</v>
       </c>
     </row>
-    <row r="102" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B102" s="7">
         <f>B91-B$100</f>
         <v>1</v>
@@ -4210,7 +4225,7 @@
         <v>2255</v>
       </c>
     </row>
-    <row r="103" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B103" s="7">
         <f t="shared" ref="B103:G103" si="10">B92-B$100</f>
         <v>-1</v>
@@ -4244,7 +4259,7 @@
         <v>705600</v>
       </c>
       <c r="K103">
-        <f t="shared" ref="K103:K107" si="13">SQRT(ABS(I103))</f>
+        <f t="shared" ref="K103:K106" si="13">SQRT(ABS(I103))</f>
         <v>28.982753492378876</v>
       </c>
       <c r="S103">
@@ -4260,7 +4275,7 @@
         <v>1805</v>
       </c>
     </row>
-    <row r="104" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B104" s="7">
         <f t="shared" ref="B104:G104" si="14">B93-B$100</f>
         <v>0</v>
@@ -4312,7 +4327,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B105" s="7">
         <f t="shared" ref="B105:G105" si="16">B94-B$100</f>
         <v>1</v>
@@ -4364,7 +4379,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="106" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B106" s="7">
         <f t="shared" ref="B106:G106" si="19">B95-B$100</f>
         <v>-1</v>
@@ -4412,7 +4427,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="107" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>79</v>
       </c>
@@ -4458,7 +4473,7 @@
         <v>0.99972295331231709</v>
       </c>
     </row>
-    <row r="108" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>80</v>
       </c>
@@ -4487,7 +4502,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="109" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B109">
         <f>(B102^2+B103^2+B104^2+B105^2+B106^2)^(1/2)</f>
         <v>2</v>
@@ -4546,7 +4561,7 @@
         <v>18.994736112934024</v>
       </c>
     </row>
-    <row r="110" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>81</v>
       </c>
@@ -4559,7 +4574,7 @@
         <v>8.9554452708952432</v>
       </c>
     </row>
-    <row r="111" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B111" s="18">
         <f>B102/B$109</f>
         <v>0.5</v>
@@ -4587,7 +4602,7 @@
         <v>-0.10241085157359611</v>
       </c>
     </row>
-    <row r="112" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B112" s="18">
         <f t="shared" ref="B112:I115" si="23">B103/B$109</f>
         <v>-0.5</v>
@@ -4633,7 +4648,7 @@
         <v>1.7888543819998317</v>
       </c>
     </row>
-    <row r="113" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B113" s="18">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -4691,7 +4706,7 @@
         <v>0.89442719099991586</v>
       </c>
     </row>
-    <row r="114" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B114" s="18">
         <f t="shared" si="23"/>
         <v>0.5</v>
@@ -4754,7 +4769,7 @@
         <v>0.44721359549995798</v>
       </c>
     </row>
-    <row r="115" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B115" s="18">
         <f t="shared" si="23"/>
         <v>-0.5</v>
@@ -4813,7 +4828,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="117" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:29" x14ac:dyDescent="0.25">
       <c r="Z117" t="s">
         <v>84</v>
       </c>
@@ -4826,7 +4841,7 @@
         <v>8.717797887081348</v>
       </c>
     </row>
-    <row r="118" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:29" x14ac:dyDescent="0.25">
       <c r="L118">
         <f>51/5</f>
         <v>10.199999999999999</v>
@@ -4876,12 +4891,12 @@
         <v>10.198039027185569</v>
       </c>
     </row>
-    <row r="120" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:29" x14ac:dyDescent="0.25">
       <c r="H120">
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:29" x14ac:dyDescent="0.25">
       <c r="H121">
         <v>5</v>
       </c>
@@ -4890,18 +4905,18 @@
         <v>45</v>
       </c>
     </row>
-    <row r="122" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:29" x14ac:dyDescent="0.25">
       <c r="H122">
         <v>10</v>
       </c>
       <c r="I122">
         <v>2</v>
       </c>
-      <c r="J122">
+      <c r="K122">
         <v>2</v>
       </c>
     </row>
-    <row r="123" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F123">
         <v>-240</v>
       </c>
@@ -4918,15 +4933,26 @@
         <v>12</v>
       </c>
       <c r="J123">
-        <f>I123/J$122</f>
+        <f>I123^2</f>
+        <v>144</v>
+      </c>
+      <c r="K123">
+        <f>I123/K$122</f>
         <v>6</v>
       </c>
-      <c r="L123">
+      <c r="M123">
         <f>2^4*3*5</f>
         <v>240</v>
       </c>
-    </row>
-    <row r="124" spans="2:29" x14ac:dyDescent="0.35">
+      <c r="N123" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="P123">
+        <f>G123/10/2</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="124" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F124">
         <v>-840</v>
       </c>
@@ -4939,19 +4965,30 @@
         <v>84</v>
       </c>
       <c r="I124">
-        <f t="shared" ref="I124:J127" si="26">$H124/I$122</f>
+        <f t="shared" ref="I124:I127" si="26">$H124/I$122</f>
         <v>42</v>
       </c>
       <c r="J124">
-        <f t="shared" ref="J124:J126" si="27">I124/J$122</f>
+        <f t="shared" ref="J124:J127" si="27">I124^2</f>
+        <v>1764</v>
+      </c>
+      <c r="K124">
+        <f>I124/K$122</f>
         <v>21</v>
       </c>
-      <c r="L124">
+      <c r="M124">
         <f>7*5*3*2^3</f>
         <v>840</v>
       </c>
-    </row>
-    <row r="125" spans="2:29" x14ac:dyDescent="0.35">
+      <c r="N124" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="P124">
+        <f>G124/10/2</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="125" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F125">
         <v>-540</v>
       </c>
@@ -4967,12 +5004,23 @@
         <f t="shared" si="26"/>
         <v>27</v>
       </c>
-      <c r="L125">
+      <c r="J125">
+        <f t="shared" si="27"/>
+        <v>729</v>
+      </c>
+      <c r="M125">
         <f>5*3^3*2^2</f>
         <v>540</v>
       </c>
-    </row>
-    <row r="126" spans="2:29" x14ac:dyDescent="0.35">
+      <c r="N125" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="P125">
+        <f>G125/10/2</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="126" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F126">
         <v>-440</v>
       </c>
@@ -4990,14 +5038,25 @@
       </c>
       <c r="J126">
         <f t="shared" si="27"/>
+        <v>484</v>
+      </c>
+      <c r="K126">
+        <f>I126/K$122</f>
         <v>11</v>
       </c>
-      <c r="L126">
+      <c r="M126">
         <f>11*5*2^3</f>
         <v>440</v>
       </c>
-    </row>
-    <row r="127" spans="2:29" x14ac:dyDescent="0.35">
+      <c r="N126" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="P126">
+        <f>G126/10/2</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="127" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F127">
         <v>2060</v>
       </c>
@@ -5013,9 +5072,115 @@
         <f t="shared" si="26"/>
         <v>103</v>
       </c>
-      <c r="L127">
+      <c r="J127">
+        <f t="shared" si="27"/>
+        <v>10609</v>
+      </c>
+      <c r="M127">
         <f>103*5*2^2</f>
         <v>2060</v>
+      </c>
+      <c r="N127" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="P127">
+        <f>G127/10/2</f>
+        <v>103</v>
+      </c>
+    </row>
+    <row r="129" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="J129">
+        <f>SUM(J123:J128)</f>
+        <v>13730</v>
+      </c>
+    </row>
+    <row r="130" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="J130">
+        <f>SQRT(J129)</f>
+        <v>117.17508267545622</v>
+      </c>
+    </row>
+    <row r="132" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F132">
+        <f>G132*H132</f>
+        <v>117</v>
+      </c>
+      <c r="G132">
+        <v>13</v>
+      </c>
+      <c r="H132">
+        <f>I132/13</f>
+        <v>9</v>
+      </c>
+      <c r="I132">
+        <v>117</v>
+      </c>
+      <c r="J132">
+        <f>I132^2</f>
+        <v>13689</v>
+      </c>
+      <c r="K132">
+        <v>41</v>
+      </c>
+      <c r="L132">
+        <f>K132+J132</f>
+        <v>13730</v>
+      </c>
+      <c r="M132">
+        <f>L132/J132</f>
+        <v>1.0029951055592081</v>
+      </c>
+      <c r="N132">
+        <f>SQRT(M132)</f>
+        <v>1.0014964331235574</v>
+      </c>
+      <c r="O132">
+        <v>2340</v>
+      </c>
+      <c r="P132">
+        <f>O132*N132</f>
+        <v>2343.5016535091245</v>
+      </c>
+    </row>
+    <row r="133" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="I133">
+        <f>I132*20</f>
+        <v>2340</v>
+      </c>
+      <c r="J133">
+        <f>J132-J129</f>
+        <v>-41</v>
+      </c>
+    </row>
+    <row r="135" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="H135">
+        <f>I135/2</f>
+        <v>59</v>
+      </c>
+      <c r="I135">
+        <v>118</v>
+      </c>
+      <c r="J135">
+        <f>I135^2</f>
+        <v>13924</v>
+      </c>
+      <c r="K135">
+        <f>J135-J129</f>
+        <v>194</v>
+      </c>
+      <c r="L135">
+        <f>K135/2</f>
+        <v>97</v>
+      </c>
+      <c r="M135">
+        <f>L135/7</f>
+        <v>13.857142857142858</v>
+      </c>
+    </row>
+    <row r="136" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="I136">
+        <f>I135*20</f>
+        <v>2360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
workings linal session task
</commit_message>
<xml_diff>
--- a/Edu/Linear_algebra/linal_session_task.xlsx
+++ b/Edu/Linear_algebra/linal_session_task.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LysogorA\DataScience\Edu\Linear_algebra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF331A3A-F6DE-41C8-BBD3-2261C83B749F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0555F8-23B6-481C-B23E-C8D5825E64DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
   </bookViews>
@@ -3073,7 +3073,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{472F5A48-0D57-45D1-AF67-58628EB4925B}">
-  <dimension ref="A1:AD136"/>
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
+  <dimension ref="A1:AD142"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="25" max="25" width="12.7109375" customWidth="1"/>
@@ -4951,6 +4954,10 @@
         <f>G123/10/2</f>
         <v>12</v>
       </c>
+      <c r="Q123">
+        <f>P123^2</f>
+        <v>144</v>
+      </c>
     </row>
     <row r="124" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F124">
@@ -4987,6 +4994,10 @@
         <f>G124/10/2</f>
         <v>42</v>
       </c>
+      <c r="Q124">
+        <f t="shared" ref="Q124:Q127" si="28">P124^2</f>
+        <v>1764</v>
+      </c>
     </row>
     <row r="125" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F125">
@@ -5019,6 +5030,10 @@
         <f>G125/10/2</f>
         <v>27</v>
       </c>
+      <c r="Q125">
+        <f t="shared" si="28"/>
+        <v>729</v>
+      </c>
     </row>
     <row r="126" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F126">
@@ -5055,6 +5070,10 @@
         <f>G126/10/2</f>
         <v>22</v>
       </c>
+      <c r="Q126">
+        <f t="shared" si="28"/>
+        <v>484</v>
+      </c>
     </row>
     <row r="127" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F127">
@@ -5087,20 +5106,66 @@
         <f>G127/10/2</f>
         <v>103</v>
       </c>
-    </row>
-    <row r="129" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="Q127">
+        <f t="shared" si="28"/>
+        <v>10609</v>
+      </c>
+    </row>
+    <row r="128" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="W128">
+        <v>2</v>
+      </c>
+      <c r="X128">
+        <f>SQRT(W128)</f>
+        <v>1.4142135623730951</v>
+      </c>
+    </row>
+    <row r="129" spans="5:24" x14ac:dyDescent="0.25">
       <c r="J129">
         <f>SUM(J123:J128)</f>
         <v>13730</v>
       </c>
-    </row>
-    <row r="130" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="P129">
+        <f>SUM(P123:P128)</f>
+        <v>206</v>
+      </c>
+      <c r="Q129">
+        <f>SUM(Q123:Q128)</f>
+        <v>13730</v>
+      </c>
+      <c r="W129">
+        <v>3</v>
+      </c>
+      <c r="X129">
+        <f>SQRT(W129)</f>
+        <v>1.7320508075688772</v>
+      </c>
+    </row>
+    <row r="130" spans="5:24" x14ac:dyDescent="0.25">
       <c r="J130">
         <f>SQRT(J129)</f>
         <v>117.17508267545622</v>
       </c>
-    </row>
-    <row r="132" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="R130">
+        <f>2*5*1373</f>
+        <v>13730</v>
+      </c>
+      <c r="S130">
+        <f>SQRT(R130)</f>
+        <v>117.17508267545622</v>
+      </c>
+    </row>
+    <row r="131" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="W131">
+        <f>W128/W129</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="X131">
+        <f>X128/X129</f>
+        <v>0.81649658092772615</v>
+      </c>
+    </row>
+    <row r="132" spans="5:24" x14ac:dyDescent="0.25">
       <c r="F132">
         <f>G132*H132</f>
         <v>117</v>
@@ -5141,8 +5206,12 @@
         <f>O132*N132</f>
         <v>2343.5016535091245</v>
       </c>
-    </row>
-    <row r="133" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="W132">
+        <f>SQRT(W131)</f>
+        <v>0.81649658092772603</v>
+      </c>
+    </row>
+    <row r="133" spans="5:24" x14ac:dyDescent="0.25">
       <c r="I133">
         <f>I132*20</f>
         <v>2340</v>
@@ -5152,7 +5221,7 @@
         <v>-41</v>
       </c>
     </row>
-    <row r="135" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="135" spans="5:24" x14ac:dyDescent="0.25">
       <c r="H135">
         <f>I135/2</f>
         <v>59</v>
@@ -5177,10 +5246,60 @@
         <v>13.857142857142858</v>
       </c>
     </row>
-    <row r="136" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="136" spans="5:24" x14ac:dyDescent="0.25">
       <c r="I136">
         <f>I135*20</f>
         <v>2360</v>
+      </c>
+    </row>
+    <row r="139" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="E139">
+        <v>19</v>
+      </c>
+      <c r="F139">
+        <v>1804</v>
+      </c>
+      <c r="H139">
+        <f>SQRT(F139/F140)*E139</f>
+        <v>18.994736112934024</v>
+      </c>
+      <c r="J139">
+        <v>9020</v>
+      </c>
+      <c r="K139">
+        <f>SQRT(J139)</f>
+        <v>94.973680564670133</v>
+      </c>
+    </row>
+    <row r="140" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="F140">
+        <v>1805</v>
+      </c>
+      <c r="J140">
+        <v>25</v>
+      </c>
+      <c r="N140">
+        <f>2 * 5 * 7 * 7 * 7 * 7</f>
+        <v>24010</v>
+      </c>
+    </row>
+    <row r="141" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="J141">
+        <f>J139/J140</f>
+        <v>360.8</v>
+      </c>
+    </row>
+    <row r="142" spans="5:24" x14ac:dyDescent="0.25">
+      <c r="M142">
+        <v>7</v>
+      </c>
+      <c r="N142">
+        <f>M142^2</f>
+        <v>49</v>
+      </c>
+      <c r="O142">
+        <f>N142^2</f>
+        <v>2401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
linal session 1 task
</commit_message>
<xml_diff>
--- a/Edu/Linear_algebra/linal_session_task.xlsx
+++ b/Edu/Linear_algebra/linal_session_task.xlsx
@@ -5,16 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iTonyJah\DataScience\Edu\Linear_algebra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LysogorA\DataScience\Edu\Linear_algebra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F698CE-2E4E-420F-9683-0F89304BC822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718BEFFB-9276-4255-8461-A2CDAF945A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" activeTab="1" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="2" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
   </bookViews>
   <sheets>
     <sheet name="calc" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="st" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="98">
   <si>
     <t>Рабочая таблица с данными:</t>
   </si>
@@ -313,13 +314,36 @@
   </si>
   <si>
     <t>меньше половины</t>
+  </si>
+  <si>
+    <t>x_1</t>
+  </si>
+  <si>
+    <t>x_2</t>
+  </si>
+  <si>
+    <t>x_3</t>
+  </si>
+  <si>
+    <t>x_4</t>
+  </si>
+  <si>
+    <t>x_5</t>
+  </si>
+  <si>
+    <t>y</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="9" x14ac:knownFonts="1">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
+  </numFmts>
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -390,8 +414,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -419,6 +450,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -485,7 +522,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -524,6 +561,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3094,18 +3137,18 @@
   <sheetPr>
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <dimension ref="A1:AD142"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AD156"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="25" max="25" width="12.7265625" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3128,7 +3171,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>3</v>
       </c>
@@ -3151,7 +3194,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1</v>
       </c>
@@ -3174,7 +3217,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>2</v>
       </c>
@@ -3197,7 +3240,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>3</v>
       </c>
@@ -3220,7 +3263,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>1</v>
       </c>
@@ -3243,32 +3286,32 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="23" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:7" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -3276,7 +3319,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>3</v>
       </c>
@@ -3290,7 +3333,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>1</v>
       </c>
@@ -3304,7 +3347,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>2</v>
       </c>
@@ -3318,22 +3361,22 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>19</v>
       </c>
@@ -3341,12 +3384,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -3354,42 +3397,42 @@
         <v>20</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="16" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="10" t="s">
         <v>28</v>
       </c>
@@ -3400,7 +3443,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="7">
         <f>F38*J$38+G38*J$39+H38*J$40</f>
         <v>93900</v>
@@ -3422,7 +3465,7 @@
       </c>
       <c r="L38" s="8"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="7">
         <f t="shared" ref="A39:A40" si="0">F39*J$38+G39*J$39+H39*J$40</f>
         <v>52100</v>
@@ -3444,7 +3487,7 @@
       </c>
       <c r="L39" s="8"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="7">
         <f t="shared" si="0"/>
         <v>80200</v>
@@ -3466,23 +3509,23 @@
       </c>
       <c r="L40" s="8"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B41" s="11" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="10"/>
       <c r="J43" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="12">
         <f>F44*J$44+G44*J$45+H44*J$46</f>
         <v>494200</v>
@@ -3504,7 +3547,7 @@
       </c>
       <c r="L44" s="8"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="12">
         <f t="shared" ref="A45:A46" si="1">F45*J$44+G45*J$45+H45*J$46</f>
         <v>9960900</v>
@@ -3526,7 +3569,7 @@
       </c>
       <c r="L45" s="8"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="12">
         <f t="shared" si="1"/>
         <v>494200</v>
@@ -3548,22 +3591,22 @@
       </c>
       <c r="L46" s="8"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B47" s="11" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B50" s="6" t="s">
         <v>43</v>
       </c>
@@ -3571,7 +3614,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="12">
         <f>$F51*J$51+$G51*J$52+$H51*J$53</f>
         <v>14</v>
@@ -3603,7 +3646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="12">
         <f t="shared" ref="A52:A53" si="4">$F52*J$51+$G52*J$52+$H52*J$53</f>
         <v>273</v>
@@ -3635,7 +3678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="12">
         <f t="shared" si="4"/>
         <v>14</v>
@@ -3667,12 +3710,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>38</v>
       </c>
@@ -3683,7 +3726,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="12">
         <f>$F51*J$51+$G51*J$52+$H51*J$53</f>
         <v>14</v>
@@ -3706,7 +3749,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="12">
         <f>$F52*J$51+$G52*J$52+$H52*J$53</f>
         <v>273</v>
@@ -3729,7 +3772,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="12">
         <f>$F53*J$51+$G53*J$52+$H53*J$53</f>
         <v>14</v>
@@ -3752,19 +3795,19 @@
         <v>48</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B59" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>51</v>
       </c>
       <c r="B60" s="8"/>
       <c r="F60" s="8"/>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G61" s="6" t="s">
         <v>43</v>
       </c>
@@ -3772,7 +3815,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="12">
         <f>F62*J$62+G62*J$63+H62*J$64</f>
         <v>494200</v>
@@ -3793,7 +3836,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="12">
         <f t="shared" ref="A63:A64" si="5">F63*J$62+G63*J$63+H63*J$64</f>
         <v>9960900</v>
@@ -3814,7 +3857,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="12">
         <f t="shared" si="5"/>
         <v>494200</v>
@@ -3835,23 +3878,23 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B65" s="11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>57</v>
       </c>
       <c r="B67" s="8"/>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C68" s="8" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="12">
         <v>494200</v>
       </c>
@@ -3859,7 +3902,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="12">
         <v>9960900</v>
       </c>
@@ -3867,7 +3910,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="12">
         <v>494200</v>
       </c>
@@ -3875,77 +3918,77 @@
         <v>59</v>
       </c>
     </row>
-    <row r="74" spans="1:3" ht="23" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" ht="23.25" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="13" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>1</v>
       </c>
@@ -3968,7 +4011,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="C90" s="16"/>
       <c r="D90" s="16"/>
       <c r="E90" s="16" t="s">
@@ -3980,7 +4023,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B91" s="7">
         <v>3</v>
       </c>
@@ -4003,7 +4046,7 @@
         <v>2200</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B92" s="7">
         <v>1</v>
       </c>
@@ -4026,7 +4069,7 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B93" s="7">
         <v>2</v>
       </c>
@@ -4049,7 +4092,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B94" s="7">
         <v>3</v>
       </c>
@@ -4072,7 +4115,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B95" s="7">
         <v>1</v>
       </c>
@@ -4095,17 +4138,17 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="97" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="13" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="98" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="99" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>76</v>
       </c>
@@ -4148,7 +4191,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="100" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>77</v>
       </c>
@@ -4185,7 +4228,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="101" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>78</v>
       </c>
@@ -4202,7 +4245,7 @@
         <v>0.44721359549995798</v>
       </c>
     </row>
-    <row r="102" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B102" s="7">
         <f>B91-B$100</f>
         <v>1</v>
@@ -4246,7 +4289,7 @@
         <v>2255</v>
       </c>
     </row>
-    <row r="103" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B103" s="7">
         <f t="shared" ref="B103:G103" si="10">B92-B$100</f>
         <v>-1</v>
@@ -4296,7 +4339,7 @@
         <v>1805</v>
       </c>
     </row>
-    <row r="104" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B104" s="7">
         <f t="shared" ref="B104:G104" si="14">B93-B$100</f>
         <v>0</v>
@@ -4348,7 +4391,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B105" s="7">
         <f t="shared" ref="B105:G105" si="16">B94-B$100</f>
         <v>1</v>
@@ -4400,7 +4443,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="106" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B106" s="7">
         <f t="shared" ref="B106:G106" si="19">B95-B$100</f>
         <v>-1</v>
@@ -4448,7 +4491,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="107" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>79</v>
       </c>
@@ -4494,7 +4537,7 @@
         <v>0.99972295331231709</v>
       </c>
     </row>
-    <row r="108" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>80</v>
       </c>
@@ -4523,7 +4566,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="109" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B109">
         <f>(B102^2+B103^2+B104^2+B105^2+B106^2)^(1/2)</f>
         <v>2</v>
@@ -4582,7 +4625,7 @@
         <v>18.994736112934024</v>
       </c>
     </row>
-    <row r="110" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>81</v>
       </c>
@@ -4595,7 +4638,7 @@
         <v>8.9554452708952432</v>
       </c>
     </row>
-    <row r="111" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B111" s="18">
         <f>B102/B$109</f>
         <v>0.5</v>
@@ -4623,7 +4666,7 @@
         <v>-0.10241085157359611</v>
       </c>
     </row>
-    <row r="112" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:30" x14ac:dyDescent="0.25">
       <c r="B112" s="18">
         <f t="shared" ref="B112:I115" si="23">B103/B$109</f>
         <v>-0.5</v>
@@ -4669,7 +4712,7 @@
         <v>1.7888543819998317</v>
       </c>
     </row>
-    <row r="113" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="113" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B113" s="18">
         <f t="shared" si="23"/>
         <v>0</v>
@@ -4727,7 +4770,7 @@
         <v>0.89442719099991586</v>
       </c>
     </row>
-    <row r="114" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="114" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B114" s="18">
         <f t="shared" si="23"/>
         <v>0.5</v>
@@ -4790,7 +4833,7 @@
         <v>0.44721359549995798</v>
       </c>
     </row>
-    <row r="115" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="115" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B115" s="18">
         <f t="shared" si="23"/>
         <v>-0.5</v>
@@ -4849,7 +4892,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="117" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="117" spans="2:29" x14ac:dyDescent="0.25">
       <c r="Z117" t="s">
         <v>84</v>
       </c>
@@ -4862,7 +4905,7 @@
         <v>8.717797887081348</v>
       </c>
     </row>
-    <row r="118" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="118" spans="2:29" x14ac:dyDescent="0.25">
       <c r="L118">
         <f>51/5</f>
         <v>10.199999999999999</v>
@@ -4912,12 +4955,12 @@
         <v>10.198039027185569</v>
       </c>
     </row>
-    <row r="120" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="120" spans="2:29" x14ac:dyDescent="0.25">
       <c r="H120">
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="121" spans="2:29" x14ac:dyDescent="0.25">
       <c r="H121">
         <v>5</v>
       </c>
@@ -4926,7 +4969,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="122" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="122" spans="2:29" x14ac:dyDescent="0.25">
       <c r="H122">
         <v>10</v>
       </c>
@@ -4937,7 +4980,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="123" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="123" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F123">
         <v>-240</v>
       </c>
@@ -4977,7 +5020,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="124" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="124" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F124">
         <v>-840</v>
       </c>
@@ -5017,7 +5060,7 @@
         <v>1764</v>
       </c>
     </row>
-    <row r="125" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="125" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F125">
         <v>-540</v>
       </c>
@@ -5053,7 +5096,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="126" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="126" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F126">
         <v>-440</v>
       </c>
@@ -5093,7 +5136,7 @@
         <v>484</v>
       </c>
     </row>
-    <row r="127" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="127" spans="2:29" x14ac:dyDescent="0.25">
       <c r="F127">
         <v>2060</v>
       </c>
@@ -5129,7 +5172,7 @@
         <v>10609</v>
       </c>
     </row>
-    <row r="128" spans="2:29" x14ac:dyDescent="0.35">
+    <row r="128" spans="2:29" x14ac:dyDescent="0.25">
       <c r="W128">
         <v>2</v>
       </c>
@@ -5138,7 +5181,7 @@
         <v>1.4142135623730951</v>
       </c>
     </row>
-    <row r="129" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="129" spans="5:24" x14ac:dyDescent="0.25">
       <c r="J129">
         <f>SUM(J123:J128)</f>
         <v>13730</v>
@@ -5159,7 +5202,7 @@
         <v>1.7320508075688772</v>
       </c>
     </row>
-    <row r="130" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="130" spans="5:24" x14ac:dyDescent="0.25">
       <c r="J130">
         <f>SQRT(J129)</f>
         <v>117.17508267545622</v>
@@ -5173,7 +5216,7 @@
         <v>117.17508267545622</v>
       </c>
     </row>
-    <row r="131" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="131" spans="5:24" x14ac:dyDescent="0.25">
       <c r="W131">
         <f>W128/W129</f>
         <v>0.66666666666666663</v>
@@ -5183,7 +5226,7 @@
         <v>0.81649658092772615</v>
       </c>
     </row>
-    <row r="132" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="132" spans="5:24" x14ac:dyDescent="0.25">
       <c r="F132">
         <f>G132*H132</f>
         <v>117</v>
@@ -5229,7 +5272,7 @@
         <v>0.81649658092772603</v>
       </c>
     </row>
-    <row r="133" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="133" spans="5:24" x14ac:dyDescent="0.25">
       <c r="I133">
         <f>I132*20</f>
         <v>2340</v>
@@ -5239,7 +5282,7 @@
         <v>-41</v>
       </c>
     </row>
-    <row r="135" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="135" spans="5:24" x14ac:dyDescent="0.25">
       <c r="H135">
         <f>I135/2</f>
         <v>59</v>
@@ -5264,13 +5307,13 @@
         <v>13.857142857142858</v>
       </c>
     </row>
-    <row r="136" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="136" spans="5:24" x14ac:dyDescent="0.25">
       <c r="I136">
         <f>I135*20</f>
         <v>2360</v>
       </c>
     </row>
-    <row r="139" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="139" spans="5:24" x14ac:dyDescent="0.25">
       <c r="E139">
         <v>19</v>
       </c>
@@ -5289,7 +5332,7 @@
         <v>94.973680564670133</v>
       </c>
     </row>
-    <row r="140" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="140" spans="5:24" x14ac:dyDescent="0.25">
       <c r="F140">
         <v>1805</v>
       </c>
@@ -5301,13 +5344,13 @@
         <v>24010</v>
       </c>
     </row>
-    <row r="141" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="141" spans="5:24" x14ac:dyDescent="0.25">
       <c r="J141">
         <f>J139/J140</f>
         <v>360.8</v>
       </c>
     </row>
-    <row r="142" spans="5:24" x14ac:dyDescent="0.35">
+    <row r="142" spans="5:24" x14ac:dyDescent="0.25">
       <c r="M142">
         <v>7</v>
       </c>
@@ -5318,6 +5361,70 @@
       <c r="O142">
         <f>N142^2</f>
         <v>2401</v>
+      </c>
+    </row>
+    <row r="148" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D148">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="149" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D149">
+        <v>5</v>
+      </c>
+      <c r="E149">
+        <f>SQRT(D149)</f>
+        <v>2.2360679774997898</v>
+      </c>
+    </row>
+    <row r="150" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="D150">
+        <f>D148/D149</f>
+        <v>0.4</v>
+      </c>
+      <c r="E150">
+        <f>D150*E149</f>
+        <v>0.89442719099991597</v>
+      </c>
+    </row>
+    <row r="151" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C151">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="152" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C152">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="153" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C153">
+        <f>C151/C152</f>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="154" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C154">
+        <f>SQRT(C153)</f>
+        <v>0.89442719099991586</v>
+      </c>
+      <c r="E154">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="155" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="E155">
+        <f>SQRT(E154)</f>
+        <v>4.4721359549995796</v>
+      </c>
+      <c r="G155">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="G156">
+        <f>G155/E155</f>
+        <v>0.22360679774997896</v>
       </c>
     </row>
   </sheetData>
@@ -5330,9 +5437,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{666D1E91-ED7C-475C-A636-9777A928839D}">
   <dimension ref="A3:O72"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
         <v>2</v>
       </c>
@@ -5359,7 +5466,7 @@
         <v>1.4310835055998654</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="11">
         <v>2</v>
       </c>
@@ -5386,9 +5493,9 @@
         <v>1.4310835055998654</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B13">
-        <f t="shared" ref="B13:B14" si="4">B14-1</f>
+        <f t="shared" ref="B13" si="4">B14-1</f>
         <v>1</v>
       </c>
       <c r="C13">
@@ -5400,9 +5507,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14">
-        <f t="shared" ref="B14:B16" si="7">B15-1</f>
+        <f t="shared" ref="B14:B15" si="7">B15-1</f>
         <v>2</v>
       </c>
       <c r="C14">
@@ -5414,7 +5521,7 @@
         <v>0.70710678118654757</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B15">
         <f t="shared" si="7"/>
         <v>3</v>
@@ -5428,7 +5535,7 @@
         <v>0.57735026918962573</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B16">
         <f>B17-1</f>
         <v>4</v>
@@ -5442,7 +5549,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>5</v>
       </c>
@@ -5455,7 +5562,7 @@
         <v>0.44721359549995798</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18">
         <f>B17+1</f>
         <v>6</v>
@@ -5469,7 +5576,7 @@
         <v>0.40824829046386296</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19">
         <f t="shared" ref="B19:B27" si="11">B18+1</f>
         <v>7</v>
@@ -5483,7 +5590,7 @@
         <v>0.37796447300922725</v>
       </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20">
         <f t="shared" si="11"/>
         <v>8</v>
@@ -5497,7 +5604,7 @@
         <v>0.35355339059327379</v>
       </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21">
         <f t="shared" si="11"/>
         <v>9</v>
@@ -5511,7 +5618,7 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22">
         <f t="shared" si="11"/>
         <v>10</v>
@@ -5525,7 +5632,7 @@
         <v>0.31622776601683794</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23">
         <f t="shared" si="11"/>
         <v>11</v>
@@ -5539,7 +5646,7 @@
         <v>0.30151134457776363</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24">
         <f t="shared" si="11"/>
         <v>12</v>
@@ -5553,7 +5660,7 @@
         <v>0.28867513459481287</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25">
         <f t="shared" si="11"/>
         <v>13</v>
@@ -5567,7 +5674,7 @@
         <v>0.27735009811261457</v>
       </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26">
         <f t="shared" si="11"/>
         <v>14</v>
@@ -5581,7 +5688,7 @@
         <v>0.2672612419124244</v>
       </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27">
         <f t="shared" si="11"/>
         <v>15</v>
@@ -5595,7 +5702,7 @@
         <v>0.25819888974716115</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28">
         <f t="shared" ref="B28:B58" si="12">B27+1</f>
         <v>16</v>
@@ -5609,7 +5716,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29">
         <f t="shared" si="12"/>
         <v>17</v>
@@ -5623,7 +5730,7 @@
         <v>0.24253562503633297</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30">
         <f t="shared" si="12"/>
         <v>18</v>
@@ -5637,7 +5744,7 @@
         <v>0.23570226039551581</v>
       </c>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31">
         <f t="shared" si="12"/>
         <v>19</v>
@@ -5651,7 +5758,7 @@
         <v>0.2294157338705618</v>
       </c>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32">
         <f t="shared" si="12"/>
         <v>20</v>
@@ -5665,7 +5772,7 @@
         <v>0.22360679774997899</v>
       </c>
     </row>
-    <row r="33" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B33">
         <f t="shared" si="12"/>
         <v>21</v>
@@ -5679,7 +5786,7 @@
         <v>0.21821789023599236</v>
       </c>
     </row>
-    <row r="34" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B34">
         <f t="shared" si="12"/>
         <v>22</v>
@@ -5693,7 +5800,7 @@
         <v>0.21320071635561044</v>
       </c>
     </row>
-    <row r="35" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B35">
         <f t="shared" si="12"/>
         <v>23</v>
@@ -5707,7 +5814,7 @@
         <v>0.20851441405707474</v>
       </c>
     </row>
-    <row r="36" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B36">
         <f t="shared" si="12"/>
         <v>24</v>
@@ -5728,7 +5835,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B37">
         <f t="shared" si="12"/>
         <v>25</v>
@@ -5757,7 +5864,7 @@
         <v>1.1180339887498949</v>
       </c>
     </row>
-    <row r="38" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B38">
         <f t="shared" si="12"/>
         <v>26</v>
@@ -5779,7 +5886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B39">
         <f t="shared" si="12"/>
         <v>27</v>
@@ -5812,7 +5919,7 @@
         <v>1.1180339887498949</v>
       </c>
     </row>
-    <row r="40" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B40">
         <f t="shared" si="12"/>
         <v>28</v>
@@ -5829,7 +5936,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B41">
         <f t="shared" si="12"/>
         <v>29</v>
@@ -5868,7 +5975,7 @@
         <v>0.22360679774997899</v>
       </c>
     </row>
-    <row r="42" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B42">
         <f t="shared" si="12"/>
         <v>30</v>
@@ -5890,7 +5997,7 @@
         <v>0.1118033988749895</v>
       </c>
     </row>
-    <row r="43" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B43">
         <f t="shared" si="12"/>
         <v>31</v>
@@ -5904,7 +6011,7 @@
         <v>0.17960530202677488</v>
       </c>
     </row>
-    <row r="44" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B44">
         <f t="shared" si="12"/>
         <v>32</v>
@@ -5927,7 +6034,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="45" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="45" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B45">
         <f t="shared" si="12"/>
         <v>33</v>
@@ -5974,7 +6081,7 @@
         <v>0.44721359549995798</v>
       </c>
     </row>
-    <row r="46" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="46" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B46">
         <f t="shared" si="12"/>
         <v>34</v>
@@ -5988,7 +6095,7 @@
         <v>0.17149858514250885</v>
       </c>
     </row>
-    <row r="47" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="47" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B47">
         <f t="shared" si="12"/>
         <v>35</v>
@@ -6005,7 +6112,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="48" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B48">
         <f t="shared" si="12"/>
         <v>36</v>
@@ -6026,7 +6133,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B49">
         <f t="shared" si="12"/>
         <v>37</v>
@@ -6046,7 +6153,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B50">
         <f t="shared" si="12"/>
         <v>38</v>
@@ -6064,7 +6171,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B51">
         <f t="shared" si="12"/>
         <v>39</v>
@@ -6082,7 +6189,7 @@
         <v>1.1180339887498949</v>
       </c>
     </row>
-    <row r="52" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B52">
         <f t="shared" si="12"/>
         <v>40</v>
@@ -6099,7 +6206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B53">
         <f t="shared" si="12"/>
         <v>41</v>
@@ -6124,7 +6231,7 @@
         <v>0.1118033988749895</v>
       </c>
     </row>
-    <row r="54" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B54">
         <f t="shared" si="12"/>
         <v>42</v>
@@ -6141,7 +6248,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="55" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B55">
         <f t="shared" si="12"/>
         <v>43</v>
@@ -6159,7 +6266,7 @@
         <v>22.360679774997898</v>
       </c>
     </row>
-    <row r="56" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B56">
         <f t="shared" si="12"/>
         <v>44</v>
@@ -6176,7 +6283,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="57" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B57">
         <f t="shared" si="12"/>
         <v>45</v>
@@ -6194,7 +6301,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="58" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B58">
         <f t="shared" si="12"/>
         <v>46</v>
@@ -6208,28 +6315,28 @@
         <v>0.14744195615489714</v>
       </c>
     </row>
-    <row r="60" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="2:10" x14ac:dyDescent="0.25">
       <c r="F60">
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="2:10" x14ac:dyDescent="0.25">
       <c r="F61">
         <f>SQRT(F60)</f>
         <v>2.8284271247461903</v>
       </c>
     </row>
-    <row r="66" spans="6:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="6:10" x14ac:dyDescent="0.25">
       <c r="G66">
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="6:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="6:10" x14ac:dyDescent="0.25">
       <c r="G67">
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="6:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F68">
         <v>2</v>
       </c>
@@ -6244,7 +6351,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="6:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="6:10" x14ac:dyDescent="0.25">
       <c r="H69">
         <f>H68/G68</f>
         <v>0.55901699437494745</v>
@@ -6258,12 +6365,12 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="71" spans="6:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F71">
         <v>80</v>
       </c>
     </row>
-    <row r="72" spans="6:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="6:10" x14ac:dyDescent="0.25">
       <c r="F72">
         <f>SQRT(F71)</f>
         <v>8.9442719099991592</v>
@@ -6279,4 +6386,794 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82BA3844-AF00-4659-9CA6-FDAA4D3C4028}">
+  <dimension ref="A2:T33"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="K2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="K3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="K4">
+        <f>K2/K3</f>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="J5">
+        <v>2</v>
+      </c>
+      <c r="K5">
+        <f>SQRT(K4)</f>
+        <v>0.89442719099991586</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <f>K5*J5</f>
+        <v>1.7888543819998317</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <f>K4</f>
+        <v>0.8</v>
+      </c>
+      <c r="K7">
+        <f>J6/K6</f>
+        <v>0.55901699437494745</v>
+      </c>
+      <c r="Q7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E8">
+        <v>1804</v>
+      </c>
+      <c r="K8">
+        <f>K7*J7</f>
+        <v>0.44721359549995798</v>
+      </c>
+      <c r="Q8">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B9" t="str">
+        <f>C17</f>
+        <v>x_1</v>
+      </c>
+      <c r="E9">
+        <v>1805</v>
+      </c>
+      <c r="F9" t="str">
+        <f>D17</f>
+        <v>x_2</v>
+      </c>
+      <c r="I9" t="str">
+        <f>E17</f>
+        <v>x_3</v>
+      </c>
+      <c r="L9" t="str">
+        <f>F17</f>
+        <v>x_4</v>
+      </c>
+      <c r="O9" t="str">
+        <f>G17</f>
+        <v>x_5</v>
+      </c>
+      <c r="Q9">
+        <v>13730</v>
+      </c>
+      <c r="R9" t="str">
+        <f>H17</f>
+        <v>y</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="E10">
+        <f>SQRT(E8/E9)</f>
+        <v>0.99972295331231709</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <v>1</v>
+      </c>
+      <c r="Q10">
+        <v>13689</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" s="7">
+        <v>1</v>
+      </c>
+      <c r="C11" s="23">
+        <f>B11*A$13</f>
+        <v>0.5</v>
+      </c>
+      <c r="E11">
+        <v>95</v>
+      </c>
+      <c r="F11" s="7">
+        <v>29</v>
+      </c>
+      <c r="G11" s="23">
+        <f>F11*E$13</f>
+        <v>0.30534775347842946</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11" s="7">
+        <v>1</v>
+      </c>
+      <c r="J11" s="23">
+        <f>I11*H$13</f>
+        <v>0.5</v>
+      </c>
+      <c r="K11">
+        <v>20</v>
+      </c>
+      <c r="L11" s="7">
+        <v>-1</v>
+      </c>
+      <c r="M11" s="23">
+        <f>L11*K$13</f>
+        <v>-0.22360679774997896</v>
+      </c>
+      <c r="N11">
+        <v>80</v>
+      </c>
+      <c r="O11" s="7">
+        <v>1</v>
+      </c>
+      <c r="P11" s="23">
+        <f>O11*N$13</f>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="Q11">
+        <f>SQRT(Q9/Q10)</f>
+        <v>1.0014964331235574</v>
+      </c>
+      <c r="R11" s="7">
+        <v>-12</v>
+      </c>
+      <c r="S11" s="23">
+        <f>R11*Q$13</f>
+        <v>-0.10241085157359613</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2</v>
+      </c>
+      <c r="B12" s="7">
+        <v>-1</v>
+      </c>
+      <c r="C12" s="23">
+        <f t="shared" ref="C12:C15" si="0">B12*A$13</f>
+        <v>-0.5</v>
+      </c>
+      <c r="E12">
+        <f>E11*E10</f>
+        <v>94.973680564670119</v>
+      </c>
+      <c r="F12" s="7">
+        <v>-76</v>
+      </c>
+      <c r="G12" s="23">
+        <f t="shared" ref="G12:G15" si="1">F12*E$13</f>
+        <v>-0.80022169877105653</v>
+      </c>
+      <c r="H12">
+        <v>2</v>
+      </c>
+      <c r="I12" s="7">
+        <v>-1</v>
+      </c>
+      <c r="J12" s="23">
+        <f t="shared" ref="J12:J15" si="2">I12*H$13</f>
+        <v>-0.5</v>
+      </c>
+      <c r="K12">
+        <f>SQRT(K11)</f>
+        <v>4.4721359549995796</v>
+      </c>
+      <c r="L12" s="7">
+        <v>-1</v>
+      </c>
+      <c r="M12" s="23">
+        <f t="shared" ref="M12:M15" si="3">L12*K$13</f>
+        <v>-0.22360679774997896</v>
+      </c>
+      <c r="N12">
+        <f>SQRT(N11)</f>
+        <v>8.9442719099991592</v>
+      </c>
+      <c r="O12" s="7">
+        <v>1</v>
+      </c>
+      <c r="P12" s="23">
+        <f t="shared" ref="P12:P15" si="4">O12*N$13</f>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="Q12">
+        <f>Q11*Q8</f>
+        <v>117.17508267545621</v>
+      </c>
+      <c r="R12" s="7">
+        <v>-42</v>
+      </c>
+      <c r="S12" s="23">
+        <f t="shared" ref="S12:S15" si="5">R12*Q$13</f>
+        <v>-0.35843798050758646</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A13" s="20">
+        <f>A11/A12</f>
+        <v>0.5</v>
+      </c>
+      <c r="B13" s="7">
+        <v>0</v>
+      </c>
+      <c r="C13" s="23">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E13" s="20">
+        <f>E7/E12</f>
+        <v>1.0529232878566533E-2</v>
+      </c>
+      <c r="F13" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G13" s="23">
+        <f t="shared" si="1"/>
+        <v>-1.0529232878566533E-2</v>
+      </c>
+      <c r="H13" s="20">
+        <f>H11/H12</f>
+        <v>0.5</v>
+      </c>
+      <c r="I13" s="7">
+        <v>0</v>
+      </c>
+      <c r="J13" s="23">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K13" s="20">
+        <f>K10/K12</f>
+        <v>0.22360679774997896</v>
+      </c>
+      <c r="L13" s="7">
+        <v>-1</v>
+      </c>
+      <c r="M13" s="23">
+        <f t="shared" si="3"/>
+        <v>-0.22360679774997896</v>
+      </c>
+      <c r="N13" s="20">
+        <f>N10/N12</f>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="O13" s="7">
+        <v>1</v>
+      </c>
+      <c r="P13" s="23">
+        <f t="shared" si="4"/>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="Q13" s="20">
+        <f>Q7/Q12</f>
+        <v>8.5342376311330105E-3</v>
+      </c>
+      <c r="R13" s="7">
+        <v>-27</v>
+      </c>
+      <c r="S13" s="23">
+        <f t="shared" si="5"/>
+        <v>-0.23042441604059127</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B14" s="7">
+        <v>1</v>
+      </c>
+      <c r="C14" s="23">
+        <f t="shared" si="0"/>
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="7">
+        <v>49</v>
+      </c>
+      <c r="G14" s="23">
+        <f t="shared" si="1"/>
+        <v>0.51593241104976018</v>
+      </c>
+      <c r="I14" s="7">
+        <v>-1</v>
+      </c>
+      <c r="J14" s="23">
+        <f t="shared" si="2"/>
+        <v>-0.5</v>
+      </c>
+      <c r="L14" s="7">
+        <v>-1</v>
+      </c>
+      <c r="M14" s="23">
+        <f t="shared" si="3"/>
+        <v>-0.22360679774997896</v>
+      </c>
+      <c r="O14" s="7">
+        <v>1</v>
+      </c>
+      <c r="P14" s="23">
+        <f t="shared" si="4"/>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="R14" s="7">
+        <v>-22</v>
+      </c>
+      <c r="S14" s="23">
+        <f t="shared" si="5"/>
+        <v>-0.18775322788492624</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B15" s="7">
+        <v>-1</v>
+      </c>
+      <c r="C15" s="23">
+        <f t="shared" si="0"/>
+        <v>-0.5</v>
+      </c>
+      <c r="F15" s="7">
+        <v>-1</v>
+      </c>
+      <c r="G15" s="23">
+        <f t="shared" si="1"/>
+        <v>-1.0529232878566533E-2</v>
+      </c>
+      <c r="I15" s="7">
+        <v>1</v>
+      </c>
+      <c r="J15" s="23">
+        <f t="shared" si="2"/>
+        <v>0.5</v>
+      </c>
+      <c r="L15" s="7">
+        <v>4</v>
+      </c>
+      <c r="M15" s="23">
+        <f t="shared" si="3"/>
+        <v>0.89442719099991586</v>
+      </c>
+      <c r="O15" s="7">
+        <v>-4</v>
+      </c>
+      <c r="P15" s="23">
+        <f t="shared" si="4"/>
+        <v>-0.44721359549995793</v>
+      </c>
+      <c r="R15" s="7">
+        <v>103</v>
+      </c>
+      <c r="S15" s="23">
+        <f t="shared" si="5"/>
+        <v>0.87902647600670003</v>
+      </c>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
+        <v>93</v>
+      </c>
+      <c r="E17" t="s">
+        <v>94</v>
+      </c>
+      <c r="F17" t="s">
+        <v>95</v>
+      </c>
+      <c r="G17" t="s">
+        <v>96</v>
+      </c>
+      <c r="H17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C19" s="24">
+        <f>C11</f>
+        <v>0.5</v>
+      </c>
+      <c r="D19" s="24">
+        <f>G11</f>
+        <v>0.30534775347842946</v>
+      </c>
+      <c r="E19" s="24">
+        <f>J11</f>
+        <v>0.5</v>
+      </c>
+      <c r="F19" s="24">
+        <f>M11</f>
+        <v>-0.22360679774997896</v>
+      </c>
+      <c r="G19" s="24">
+        <f>P11</f>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="H19" s="24">
+        <f>S11</f>
+        <v>-0.10241085157359613</v>
+      </c>
+      <c r="J19" t="str">
+        <f>C19&amp;" &amp; "&amp;D19</f>
+        <v>0.5 &amp; 0.305347753478429</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C20" s="24">
+        <f t="shared" ref="C20:C23" si="6">C12</f>
+        <v>-0.5</v>
+      </c>
+      <c r="D20" s="24">
+        <f t="shared" ref="D20:D23" si="7">G12</f>
+        <v>-0.80022169877105653</v>
+      </c>
+      <c r="E20" s="24">
+        <f t="shared" ref="E20:E23" si="8">J12</f>
+        <v>-0.5</v>
+      </c>
+      <c r="F20" s="24">
+        <f t="shared" ref="F20:F23" si="9">M12</f>
+        <v>-0.22360679774997896</v>
+      </c>
+      <c r="G20" s="24">
+        <f t="shared" ref="G20:G23" si="10">P12</f>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="H20" s="24">
+        <f t="shared" ref="H20:H23" si="11">S12</f>
+        <v>-0.35843798050758646</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C21" s="24">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="D21" s="24">
+        <f t="shared" si="7"/>
+        <v>-1.0529232878566533E-2</v>
+      </c>
+      <c r="E21" s="24">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F21" s="24">
+        <f t="shared" si="9"/>
+        <v>-0.22360679774997896</v>
+      </c>
+      <c r="G21" s="24">
+        <f t="shared" si="10"/>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="H21" s="24">
+        <f t="shared" si="11"/>
+        <v>-0.23042441604059127</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C22" s="24">
+        <f t="shared" si="6"/>
+        <v>0.5</v>
+      </c>
+      <c r="D22" s="24">
+        <f t="shared" si="7"/>
+        <v>0.51593241104976018</v>
+      </c>
+      <c r="E22" s="24">
+        <f t="shared" si="8"/>
+        <v>-0.5</v>
+      </c>
+      <c r="F22" s="24">
+        <f t="shared" si="9"/>
+        <v>-0.22360679774997896</v>
+      </c>
+      <c r="G22" s="24">
+        <f t="shared" si="10"/>
+        <v>0.11180339887498948</v>
+      </c>
+      <c r="H22" s="24">
+        <f t="shared" si="11"/>
+        <v>-0.18775322788492624</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C23" s="24">
+        <f t="shared" si="6"/>
+        <v>-0.5</v>
+      </c>
+      <c r="D23" s="24">
+        <f t="shared" si="7"/>
+        <v>-1.0529232878566533E-2</v>
+      </c>
+      <c r="E23" s="24">
+        <f t="shared" si="8"/>
+        <v>0.5</v>
+      </c>
+      <c r="F23" s="24">
+        <f t="shared" si="9"/>
+        <v>0.89442719099991586</v>
+      </c>
+      <c r="G23" s="24">
+        <f t="shared" si="10"/>
+        <v>-0.44721359549995793</v>
+      </c>
+      <c r="H23" s="24">
+        <f t="shared" si="11"/>
+        <v>0.87902647600670003</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C24" s="22"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="22"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="S24">
+        <f>1/5</f>
+        <v>0.2</v>
+      </c>
+      <c r="T24">
+        <f>0-S24</f>
+        <v>-0.2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C25" s="22">
+        <f>SUM(C19:C24)</f>
+        <v>0</v>
+      </c>
+      <c r="D25" s="22">
+        <f t="shared" ref="D25:H25" si="12">SUM(D19:D24)</f>
+        <v>1.9081958235744878E-17</v>
+      </c>
+      <c r="E25" s="22">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="F25" s="22">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G25" s="22">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="H25" s="22">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="R26">
+        <f>4/5</f>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A27" s="26">
+        <v>4</v>
+      </c>
+      <c r="C27" s="25">
+        <f>ROUND(C19,$A$27)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D27" s="25">
+        <f t="shared" ref="D27:H27" si="13">ROUND(D19,$A$27)</f>
+        <v>0.30530000000000002</v>
+      </c>
+      <c r="E27" s="25">
+        <f t="shared" si="13"/>
+        <v>0.5</v>
+      </c>
+      <c r="F27" s="25">
+        <f t="shared" si="13"/>
+        <v>-0.22359999999999999</v>
+      </c>
+      <c r="G27" s="25">
+        <f t="shared" si="13"/>
+        <v>0.1118</v>
+      </c>
+      <c r="H27" s="25">
+        <f t="shared" si="13"/>
+        <v>-0.1024</v>
+      </c>
+      <c r="J27" t="str">
+        <f>C27&amp;" &amp; "&amp;D27&amp;" &amp; "&amp;E27&amp;" &amp; "&amp;F27&amp;" &amp; "&amp;G27&amp;" &amp; "&amp;H27</f>
+        <v>0.5 &amp; 0.3053 &amp; 0.5 &amp; -0.2236 &amp; 0.1118 &amp; -0.1024</v>
+      </c>
+      <c r="R27">
+        <f>R26/S24</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C28" s="25">
+        <f t="shared" ref="C28:H28" si="14">ROUND(C20,$A$27)</f>
+        <v>-0.5</v>
+      </c>
+      <c r="D28" s="25">
+        <f t="shared" si="14"/>
+        <v>-0.80020000000000002</v>
+      </c>
+      <c r="E28" s="25">
+        <f t="shared" si="14"/>
+        <v>-0.5</v>
+      </c>
+      <c r="F28" s="25">
+        <f t="shared" si="14"/>
+        <v>-0.22359999999999999</v>
+      </c>
+      <c r="G28" s="25">
+        <f t="shared" si="14"/>
+        <v>0.1118</v>
+      </c>
+      <c r="H28" s="25">
+        <f t="shared" si="14"/>
+        <v>-0.3584</v>
+      </c>
+      <c r="J28" t="str">
+        <f t="shared" ref="J28:J31" si="15">C28&amp;" &amp; "&amp;D28&amp;" &amp; "&amp;E28&amp;" &amp; "&amp;F28&amp;" &amp; "&amp;G28&amp;" &amp; "&amp;H28</f>
+        <v>-0.5 &amp; -0.8002 &amp; -0.5 &amp; -0.2236 &amp; 0.1118 &amp; -0.3584</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C29" s="25">
+        <f t="shared" ref="C29:H29" si="16">ROUND(C21,$A$27)</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="25">
+        <f t="shared" si="16"/>
+        <v>-1.0500000000000001E-2</v>
+      </c>
+      <c r="E29" s="25">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="F29" s="25">
+        <f t="shared" si="16"/>
+        <v>-0.22359999999999999</v>
+      </c>
+      <c r="G29" s="25">
+        <f t="shared" si="16"/>
+        <v>0.1118</v>
+      </c>
+      <c r="H29" s="25">
+        <f t="shared" si="16"/>
+        <v>-0.23039999999999999</v>
+      </c>
+      <c r="J29" t="str">
+        <f t="shared" si="15"/>
+        <v>0 &amp; -0.0105 &amp; 0 &amp; -0.2236 &amp; 0.1118 &amp; -0.2304</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C30" s="25">
+        <f t="shared" ref="C30:H30" si="17">ROUND(C22,$A$27)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D30" s="25">
+        <f t="shared" si="17"/>
+        <v>0.51590000000000003</v>
+      </c>
+      <c r="E30" s="25">
+        <f t="shared" si="17"/>
+        <v>-0.5</v>
+      </c>
+      <c r="F30" s="25">
+        <f t="shared" si="17"/>
+        <v>-0.22359999999999999</v>
+      </c>
+      <c r="G30" s="25">
+        <f t="shared" si="17"/>
+        <v>0.1118</v>
+      </c>
+      <c r="H30" s="25">
+        <f t="shared" si="17"/>
+        <v>-0.18779999999999999</v>
+      </c>
+      <c r="J30" t="str">
+        <f t="shared" si="15"/>
+        <v>0.5 &amp; 0.5159 &amp; -0.5 &amp; -0.2236 &amp; 0.1118 &amp; -0.1878</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="C31" s="25">
+        <f t="shared" ref="C31:H31" si="18">ROUND(C23,$A$27)</f>
+        <v>-0.5</v>
+      </c>
+      <c r="D31" s="25">
+        <f t="shared" si="18"/>
+        <v>-1.0500000000000001E-2</v>
+      </c>
+      <c r="E31" s="25">
+        <f t="shared" si="18"/>
+        <v>0.5</v>
+      </c>
+      <c r="F31" s="25">
+        <f t="shared" si="18"/>
+        <v>0.89439999999999997</v>
+      </c>
+      <c r="G31" s="25">
+        <f t="shared" si="18"/>
+        <v>-0.44719999999999999</v>
+      </c>
+      <c r="H31" s="25">
+        <f t="shared" si="18"/>
+        <v>0.879</v>
+      </c>
+      <c r="J31" t="str">
+        <f t="shared" si="15"/>
+        <v>-0.5 &amp; -0.0105 &amp; 0.5 &amp; 0.8944 &amp; -0.4472 &amp; 0.879</v>
+      </c>
+    </row>
+    <row r="33" spans="3:8" x14ac:dyDescent="0.25">
+      <c r="C33" s="27">
+        <f>SUM(C27:C32)</f>
+        <v>0</v>
+      </c>
+      <c r="D33" s="27">
+        <f t="shared" ref="D33:H33" si="19">SUM(D27:D32)</f>
+        <v>6.4184768611141862E-17</v>
+      </c>
+      <c r="E33" s="27">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="F33" s="27">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="G33" s="27">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+      <c r="H33" s="27">
+        <f t="shared" si="19"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="9" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
linal session task, py_base session task
</commit_message>
<xml_diff>
--- a/Edu/Linear_algebra/linal_session_task.xlsx
+++ b/Edu/Linear_algebra/linal_session_task.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LysogorA\DataScience\Edu\Linear_algebra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D03A45-8DE2-4F8B-AB00-D5DDE8DC62E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74A692C3-DADE-4900-B0BC-8FD14E0A5956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{6B48EADF-CD2A-4593-B5B4-C8A55DF2A88B}"/>
   </bookViews>
   <sheets>
     <sheet name="calc" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
-    <sheet name="st" sheetId="3" r:id="rId3"/>
+    <sheet name="split1" sheetId="4" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId3"/>
+    <sheet name="st" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="105">
   <si>
     <t>Рабочая таблица с данными:</t>
   </si>
@@ -332,6 +333,27 @@
   </si>
   <si>
     <t>y</t>
+  </si>
+  <si>
+    <t>среднее</t>
+  </si>
+  <si>
+    <t>центрированые</t>
+  </si>
+  <si>
+    <t>длина ц.в.</t>
+  </si>
+  <si>
+    <t>standart</t>
+  </si>
+  <si>
+    <t>check</t>
+  </si>
+  <si>
+    <t>Спальный</t>
+  </si>
+  <si>
+    <t>Центральный</t>
   </si>
 </sst>
 </file>
@@ -545,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -594,6 +616,7 @@
     <xf numFmtId="165" fontId="10" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5462,6 +5485,556 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{187E156B-4495-4400-8873-A45B82A27CF2}">
+  <dimension ref="B1:L28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
+      <c r="F2" s="9"/>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C3" s="7">
+        <v>3</v>
+      </c>
+      <c r="D3" s="7">
+        <v>51</v>
+      </c>
+      <c r="E3" s="7">
+        <v>3</v>
+      </c>
+      <c r="F3" s="7">
+        <v>2200</v>
+      </c>
+      <c r="H3" s="7">
+        <v>1</v>
+      </c>
+      <c r="I3" s="7">
+        <v>45</v>
+      </c>
+      <c r="J3" s="7">
+        <v>3</v>
+      </c>
+      <c r="K3" s="7">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C4" s="7">
+        <v>1</v>
+      </c>
+      <c r="D4" s="7">
+        <v>30</v>
+      </c>
+      <c r="E4" s="7">
+        <v>1</v>
+      </c>
+      <c r="F4" s="7">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C5" s="7">
+        <v>2</v>
+      </c>
+      <c r="D5" s="7">
+        <v>45</v>
+      </c>
+      <c r="E5" s="7">
+        <v>2</v>
+      </c>
+      <c r="F5" s="7">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C6" s="7">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7">
+        <v>55</v>
+      </c>
+      <c r="E6" s="7">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8">
+        <f>AVERAGE(C3:C6)</f>
+        <v>2.25</v>
+      </c>
+      <c r="D8">
+        <f t="shared" ref="D8:F8" si="0">AVERAGE(D3:D6)</f>
+        <v>45.25</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>1.75</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>1925</v>
+      </c>
+      <c r="H8">
+        <f>AVERAGE(H3:H6)</f>
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <f t="shared" ref="I8:K8" si="1">AVERAGE(I3:I6)</f>
+        <v>45</v>
+      </c>
+      <c r="J8">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="1"/>
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10">
+        <f>C3-C$8</f>
+        <v>0.75</v>
+      </c>
+      <c r="D10">
+        <f t="shared" ref="D10:F10" si="2">D3-D$8</f>
+        <v>5.75</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="2"/>
+        <v>1.25</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="2"/>
+        <v>275</v>
+      </c>
+      <c r="H10">
+        <f>H3-H$8</f>
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <f t="shared" ref="I10:K10" si="3">I3-I$8</f>
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C11">
+        <f t="shared" ref="C11:F11" si="4">C4-C$8</f>
+        <v>-1.25</v>
+      </c>
+      <c r="D11">
+        <f t="shared" si="4"/>
+        <v>-15.25</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="4"/>
+        <v>-0.75</v>
+      </c>
+      <c r="F11">
+        <f t="shared" si="4"/>
+        <v>-325</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C12">
+        <f t="shared" ref="C12:F12" si="5">C5-C$8</f>
+        <v>-0.25</v>
+      </c>
+      <c r="D12">
+        <f t="shared" si="5"/>
+        <v>-0.25</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="5"/>
+        <v>0.25</v>
+      </c>
+      <c r="F12">
+        <f t="shared" si="5"/>
+        <v>-25</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C13">
+        <f t="shared" ref="C13:F13" si="6">C6-C$8</f>
+        <v>0.75</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="6"/>
+        <v>9.75</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="6"/>
+        <v>-0.75</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="6"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <f>C10^2</f>
+        <v>0.5625</v>
+      </c>
+      <c r="D15">
+        <f t="shared" ref="D15:F15" si="7">D10^2</f>
+        <v>33.0625</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="7"/>
+        <v>1.5625</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="7"/>
+        <v>75625</v>
+      </c>
+      <c r="H15">
+        <f>H10^2</f>
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <f t="shared" ref="I15:K15" si="8">I10^2</f>
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="C16">
+        <f t="shared" ref="C16:F16" si="9">C11^2</f>
+        <v>1.5625</v>
+      </c>
+      <c r="D16">
+        <f t="shared" si="9"/>
+        <v>232.5625</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="9"/>
+        <v>0.5625</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="9"/>
+        <v>105625</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C17">
+        <f t="shared" ref="C17:F17" si="10">C12^2</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="10"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="10"/>
+        <v>6.25E-2</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="10"/>
+        <v>625</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C18">
+        <f t="shared" ref="C18:F18" si="11">C13^2</f>
+        <v>0.5625</v>
+      </c>
+      <c r="D18">
+        <f t="shared" si="11"/>
+        <v>95.0625</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="11"/>
+        <v>0.5625</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="11"/>
+        <v>5625</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C20">
+        <f>SUM(C15:C19)</f>
+        <v>2.75</v>
+      </c>
+      <c r="D20">
+        <f t="shared" ref="D20:F20" si="12">SUM(D15:D19)</f>
+        <v>360.75</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="12"/>
+        <v>2.75</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="12"/>
+        <v>187500</v>
+      </c>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C21">
+        <f>SQRT(C20)</f>
+        <v>1.6583123951776999</v>
+      </c>
+      <c r="D21">
+        <f t="shared" ref="D21:F21" si="13">SQRT(D20)</f>
+        <v>18.993419913222578</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="13"/>
+        <v>1.6583123951776999</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="13"/>
+        <v>433.0127018922193</v>
+      </c>
+    </row>
+    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>101</v>
+      </c>
+      <c r="C23" s="32">
+        <f>C10/C$21</f>
+        <v>0.45226701686664544</v>
+      </c>
+      <c r="D23" s="32">
+        <f t="shared" ref="D23:F23" si="14">D10/D$21</f>
+        <v>0.30273642273327744</v>
+      </c>
+      <c r="E23" s="32">
+        <f t="shared" si="14"/>
+        <v>0.75377836144440902</v>
+      </c>
+      <c r="F23" s="32">
+        <f t="shared" si="14"/>
+        <v>0.63508529610858833</v>
+      </c>
+      <c r="G23" s="32"/>
+      <c r="H23" s="32">
+        <f>C23*$F23</f>
+        <v>0.28722813232690142</v>
+      </c>
+      <c r="I23" s="32">
+        <f t="shared" ref="I23:K23" si="15">D23*$F23</f>
+        <v>0.19226345067441827</v>
+      </c>
+      <c r="J23" s="32">
+        <f t="shared" si="15"/>
+        <v>0.478713553878169</v>
+      </c>
+      <c r="K23" s="32">
+        <f t="shared" si="15"/>
+        <v>0.40333333333333332</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="32">
+        <f t="shared" ref="C24:F26" si="16">C11/C$21</f>
+        <v>-0.75377836144440902</v>
+      </c>
+      <c r="D24" s="32">
+        <f t="shared" si="16"/>
+        <v>-0.80290964290130107</v>
+      </c>
+      <c r="E24" s="32">
+        <f t="shared" si="16"/>
+        <v>-0.45226701686664544</v>
+      </c>
+      <c r="F24" s="32">
+        <f t="shared" si="16"/>
+        <v>-0.75055534994651352</v>
+      </c>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32">
+        <f t="shared" ref="H24:H26" si="17">C24*$F24</f>
+        <v>0.56575238185601795</v>
+      </c>
+      <c r="I24" s="32">
+        <f t="shared" ref="I24:I26" si="18">D24*$F24</f>
+        <v>0.60262812800321619</v>
+      </c>
+      <c r="J24" s="32">
+        <f t="shared" ref="J24:J26" si="19">E24*$F24</f>
+        <v>0.33945142911361081</v>
+      </c>
+      <c r="K24" s="32">
+        <f t="shared" ref="K24:K26" si="20">F24*$F24</f>
+        <v>0.56333333333333335</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="32">
+        <f t="shared" si="16"/>
+        <v>-0.15075567228888181</v>
+      </c>
+      <c r="D25" s="32">
+        <f t="shared" si="16"/>
+        <v>-1.316245316231641E-2</v>
+      </c>
+      <c r="E25" s="32">
+        <f t="shared" si="16"/>
+        <v>0.15075567228888181</v>
+      </c>
+      <c r="F25" s="32">
+        <f t="shared" si="16"/>
+        <v>-5.7735026918962581E-2</v>
+      </c>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32">
+        <f t="shared" si="17"/>
+        <v>8.7038827977848933E-3</v>
+      </c>
+      <c r="I25" s="32">
+        <f t="shared" si="18"/>
+        <v>7.5993458764592203E-4</v>
+      </c>
+      <c r="J25" s="32">
+        <f t="shared" si="19"/>
+        <v>-8.7038827977848933E-3</v>
+      </c>
+      <c r="K25" s="32">
+        <f t="shared" si="20"/>
+        <v>3.333333333333334E-3</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C26" s="32">
+        <f t="shared" si="16"/>
+        <v>0.45226701686664544</v>
+      </c>
+      <c r="D26" s="32">
+        <f t="shared" si="16"/>
+        <v>0.51333567333034003</v>
+      </c>
+      <c r="E26" s="32">
+        <f t="shared" si="16"/>
+        <v>-0.45226701686664544</v>
+      </c>
+      <c r="F26" s="32">
+        <f t="shared" si="16"/>
+        <v>0.17320508075688773</v>
+      </c>
+      <c r="G26" s="32"/>
+      <c r="H26" s="32">
+        <f t="shared" si="17"/>
+        <v>7.8334945180064036E-2</v>
+      </c>
+      <c r="I26" s="32">
+        <f t="shared" si="18"/>
+        <v>8.891234675457288E-2</v>
+      </c>
+      <c r="J26" s="32">
+        <f t="shared" si="19"/>
+        <v>-7.8334945180064036E-2</v>
+      </c>
+      <c r="K26" s="32">
+        <f t="shared" si="20"/>
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C27" s="32"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="32"/>
+      <c r="G27" s="32"/>
+      <c r="H27" s="32"/>
+      <c r="I27" s="32"/>
+      <c r="J27" s="32"/>
+      <c r="K27" s="32"/>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>102</v>
+      </c>
+      <c r="C28" s="32">
+        <f>SUM(C23:C27)</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="32">
+        <f t="shared" ref="D28:F28" si="21">SUM(D23:D27)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="32">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="F28" s="32">
+        <f t="shared" si="21"/>
+        <v>0</v>
+      </c>
+      <c r="G28" s="32"/>
+      <c r="H28" s="32">
+        <f t="shared" ref="H28" si="22">SUM(H23:H27)</f>
+        <v>0.94001934216076832</v>
+      </c>
+      <c r="I28" s="32">
+        <f t="shared" ref="I28" si="23">SUM(I23:I27)</f>
+        <v>0.88456386001985332</v>
+      </c>
+      <c r="J28" s="32">
+        <f t="shared" ref="J28" si="24">SUM(J23:J27)</f>
+        <v>0.73112615501393097</v>
+      </c>
+      <c r="K28" s="32">
+        <f t="shared" ref="K28" si="25">SUM(K23:K27)</f>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{666D1E91-ED7C-475C-A636-9777A928839D}">
   <dimension ref="A3:O72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6415,7 +6988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82BA3844-AF00-4659-9CA6-FDAA4D3C4028}">
   <dimension ref="A2:T83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -8090,7 +8663,7 @@
         <v>0.01</v>
       </c>
       <c r="Q77" t="str">
-        <f t="shared" ref="Q77:Q83" si="34">J77&amp;" &amp; "&amp;K77&amp;" &amp; "&amp;L77&amp;" &amp; "&amp;M77&amp;" &amp; "&amp;N77&amp;" &amp; "&amp;O77</f>
+        <f t="shared" ref="Q77:Q81" si="34">J77&amp;" &amp; "&amp;K77&amp;" &amp; "&amp;L77&amp;" &amp; "&amp;M77&amp;" &amp; "&amp;N77&amp;" &amp; "&amp;O77</f>
         <v>-0.05 &amp; -0.03 &amp; -0.05 &amp; 0.02 &amp; -0.01 &amp; 0.01</v>
       </c>
     </row>

</xml_diff>